<commit_message>
chore(resources): sync bundled input_template.xlsx from v16 master
Byte-copy of the committed v16 master (docs/inputs/input_template.xlsx @8a16762).
Keeps the wheel copy identical to the editable docs master, as the template_sync
guard requires.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/xslope/resources/input_template.xlsx
+++ b/xslope/resources/input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E95D610-588A-C249-B900-E3D88174AD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448736C4-E2C8-EB41-827A-888C500BCAB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="238">
   <si>
     <t>X</t>
   </si>
@@ -305,9 +305,6 @@
     <t>s(f)</t>
   </si>
   <si>
-    <t>Base Values</t>
-  </si>
-  <si>
     <t>Standard Deviations</t>
   </si>
   <si>
@@ -460,9 +457,6 @@
   </si>
   <si>
     <t>XSLOPE Input Template</t>
-  </si>
-  <si>
-    <t>Stress</t>
   </si>
   <si>
     <t>E</t>
@@ -932,6 +926,21 @@
   </si>
   <si>
     <t>Line loads</t>
+  </si>
+  <si>
+    <t>elastic</t>
+  </si>
+  <si>
+    <t>Elastic / infinite strength (cannot fail). FEM: no yield; LEM: impenetrable</t>
+  </si>
+  <si>
+    <t>t_cut</t>
+  </si>
+  <si>
+    <t>Shear Strength/Stiffness</t>
+  </si>
+  <si>
+    <t>Color legend</t>
   </si>
 </sst>
 </file>
@@ -1081,7 +1090,7 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1144,12 +1153,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1175,6 +1178,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1265,7 +1280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1322,26 +1337,14 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1360,28 +1363,28 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1394,13 +1397,16 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1410,12 +1416,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1433,8 +1433,32 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10394,7 +10418,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="32" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="19" x14ac:dyDescent="0.25">
@@ -10404,22 +10428,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="34">
-        <v>15</v>
+        <v>78</v>
+      </c>
+      <c r="D5" s="30">
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="49" t="s">
+      <c r="B7" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="35" t="s">
+      <c r="G7" s="31" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10431,10 +10455,10 @@
         <v>62.4</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -10468,16 +10492,16 @@
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B11" s="1"/>
       <c r="C11" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D11" s="1">
         <v>0</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="G11" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -10514,10 +10538,10 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F16" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G16" t="s">
         <v>117</v>
-      </c>
-      <c r="G16" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
@@ -10531,34 +10555,34 @@
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F18" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="G18" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F19" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="G19" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F20" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F21" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="G21" s="9" t="s">
         <v>118</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
@@ -10595,36 +10619,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="54" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="F2" s="54" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="J2" s="54" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="F2" s="59" t="s">
+      <c r="K2" s="54"/>
+      <c r="L2" s="54"/>
+      <c r="N2" s="54" t="s">
         <v>132</v>
       </c>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="J2" s="59" t="s">
+      <c r="O2" s="54"/>
+      <c r="P2" s="54"/>
+      <c r="R2" s="54" t="s">
         <v>133</v>
       </c>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="N2" s="59" t="s">
+      <c r="S2" s="54"/>
+      <c r="T2" s="54"/>
+      <c r="V2" s="54" t="s">
         <v>134</v>
       </c>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="R2" s="59" t="s">
-        <v>135</v>
-      </c>
-      <c r="S2" s="59"/>
-      <c r="T2" s="59"/>
-      <c r="V2" s="59" t="s">
-        <v>136</v>
-      </c>
-      <c r="W2" s="59"/>
-      <c r="X2" s="59"/>
+      <c r="W2" s="54"/>
+      <c r="X2" s="54"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -11093,64 +11117,64 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C2" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="G2" s="40" t="s">
+        <v>192</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>193</v>
+      </c>
+      <c r="I2" s="40" t="s">
+        <v>177</v>
+      </c>
+      <c r="J2" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="K2" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="L2" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="M2" s="27" t="s">
+        <v>178</v>
+      </c>
+      <c r="N2" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="O2" s="27" t="s">
+        <v>194</v>
+      </c>
+      <c r="P2" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q2" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="R2" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="F2" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="G2" s="44" t="s">
-        <v>194</v>
-      </c>
-      <c r="H2" s="44" t="s">
-        <v>195</v>
-      </c>
-      <c r="I2" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="J2" s="31" t="s">
-        <v>106</v>
-      </c>
-      <c r="K2" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="L2" s="31" t="s">
-        <v>108</v>
-      </c>
-      <c r="M2" s="31" t="s">
+      <c r="Z2" t="s">
         <v>180</v>
       </c>
-      <c r="N2" s="31" t="s">
+      <c r="AA2" t="s">
         <v>181</v>
       </c>
-      <c r="O2" s="31" t="s">
-        <v>196</v>
-      </c>
-      <c r="P2" s="32" t="s">
-        <v>109</v>
-      </c>
-      <c r="Q2" s="32" t="s">
-        <v>99</v>
-      </c>
-      <c r="R2" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="Z2" t="s">
+      <c r="AB2" t="s">
         <v>182</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>183</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
@@ -11181,13 +11205,13 @@
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
       <c r="Z3" t="s">
+        <v>183</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>184</v>
+      </c>
+      <c r="AB3" t="s">
         <v>185</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>186</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.2">
@@ -11218,7 +11242,7 @@
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
       <c r="Z4" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
@@ -11249,7 +11273,7 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="Z5" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -11336,13 +11360,13 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
       <c r="Z8" t="s">
+        <v>180</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>181</v>
+      </c>
+      <c r="AB8" t="s">
         <v>182</v>
-      </c>
-      <c r="AA8" t="s">
-        <v>183</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
@@ -11373,13 +11397,13 @@
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
       <c r="Z9" t="s">
+        <v>183</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>184</v>
+      </c>
+      <c r="AB9" t="s">
         <v>185</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>186</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
@@ -11410,13 +11434,13 @@
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
       <c r="Z10" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="AA10" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="AB10" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
@@ -11447,13 +11471,13 @@
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
       <c r="Z11" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="AA11" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="AB11" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
@@ -11765,25 +11789,25 @@
       <c r="R22" s="3"/>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="T23" s="46"/>
+      <c r="T23" s="42"/>
       <c r="U23" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
-      <c r="T24" s="30"/>
+      <c r="T24" s="26"/>
       <c r="U24" s="9" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.2">
       <c r="K25" s="9"/>
       <c r="L25" s="9"/>
-      <c r="T25" s="33"/>
+      <c r="T25" s="29"/>
       <c r="U25" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -11821,58 +11845,58 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C2" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="G2" s="40" t="s">
+        <v>152</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="I2" s="40" t="s">
+        <v>177</v>
+      </c>
+      <c r="J2" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="K2" s="27" t="s">
+        <v>154</v>
+      </c>
+      <c r="L2" s="41" t="s">
+        <v>157</v>
+      </c>
+      <c r="M2" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="N2" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="O2" s="28" t="s">
+        <v>155</v>
+      </c>
+      <c r="P2" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="F2" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="G2" s="44" t="s">
-        <v>154</v>
-      </c>
-      <c r="H2" s="44" t="s">
-        <v>162</v>
-      </c>
-      <c r="I2" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="J2" s="31" t="s">
-        <v>155</v>
-      </c>
-      <c r="K2" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="L2" s="45" t="s">
-        <v>159</v>
-      </c>
-      <c r="M2" s="45" t="s">
-        <v>160</v>
-      </c>
-      <c r="N2" s="32" t="s">
-        <v>99</v>
-      </c>
-      <c r="O2" s="32" t="s">
-        <v>157</v>
-      </c>
-      <c r="P2" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q2" s="32" t="s">
-        <v>166</v>
+      <c r="Q2" s="28" t="s">
+        <v>164</v>
       </c>
       <c r="Z2" t="s">
         <v>40</v>
       </c>
       <c r="AA2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
@@ -11896,10 +11920,10 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="Z3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AA3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
@@ -12100,21 +12124,21 @@
       <c r="K15" s="9"/>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="S16" s="46"/>
+      <c r="S16" s="42"/>
       <c r="T16" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" spans="19:20" x14ac:dyDescent="0.2">
+      <c r="S17" s="26"/>
+      <c r="T17" s="9" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="18" spans="19:20" x14ac:dyDescent="0.2">
+      <c r="S18" s="29"/>
+      <c r="T18" s="9" t="s">
         <v>163</v>
-      </c>
-    </row>
-    <row r="17" spans="19:20" x14ac:dyDescent="0.2">
-      <c r="S17" s="30"/>
-      <c r="T17" s="9" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="18" spans="19:20" x14ac:dyDescent="0.2">
-      <c r="S18" s="33"/>
-      <c r="T18" s="9" t="s">
-        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -12146,7 +12170,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C2" s="12" t="s">
         <v>3</v>
@@ -12155,10 +12179,10 @@
         <v>4</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -12380,100 +12404,100 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="60" t="s">
-        <v>129</v>
-      </c>
-      <c r="C2" s="60"/>
-      <c r="E2" s="56" t="s">
+      <c r="B2" s="55" t="s">
+        <v>127</v>
+      </c>
+      <c r="C2" s="55"/>
+      <c r="E2" s="51" t="s">
+        <v>215</v>
+      </c>
+      <c r="F2" s="51"/>
+      <c r="H2" s="51" t="s">
         <v>217</v>
       </c>
-      <c r="F2" s="56"/>
-      <c r="H2" s="56" t="s">
+      <c r="I2" s="51"/>
+      <c r="K2" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="L2" s="51"/>
+      <c r="N2" s="51" t="s">
         <v>219</v>
       </c>
-      <c r="I2" s="56"/>
-      <c r="K2" s="56" t="s">
+      <c r="O2" s="51"/>
+      <c r="Q2" s="51" t="s">
         <v>220</v>
       </c>
-      <c r="L2" s="56"/>
-      <c r="N2" s="56" t="s">
-        <v>221</v>
-      </c>
-      <c r="O2" s="56"/>
-      <c r="Q2" s="56" t="s">
-        <v>222</v>
-      </c>
-      <c r="R2" s="56"/>
+      <c r="R2" s="51"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="E3" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="F3" s="37"/>
-      <c r="H3" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="I3" s="37"/>
-      <c r="K3" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="L3" s="37"/>
-      <c r="N3" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="O3" s="37"/>
-      <c r="Q3" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="R3" s="37"/>
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="E3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="33"/>
+      <c r="H3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="I3" s="33"/>
+      <c r="K3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="L3" s="33"/>
+      <c r="N3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="O3" s="33"/>
+      <c r="Q3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="R3" s="33"/>
       <c r="T3" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="28" t="s">
+      <c r="E4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="28" t="s">
+      <c r="H4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="28" t="s">
+      <c r="I4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="28" t="s">
+      <c r="K4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="L4" s="28" t="s">
+      <c r="L4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="28" t="s">
+      <c r="N4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="O4" s="28" t="s">
+      <c r="O4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="Q4" s="28" t="s">
+      <c r="Q4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="R4" s="28" t="s">
+      <c r="R4" s="25" t="s">
         <v>4</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="U4" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -12490,10 +12514,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="U5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -12796,100 +12820,100 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="61" t="s">
-        <v>130</v>
-      </c>
-      <c r="C2" s="61"/>
-      <c r="E2" s="57" t="s">
+      <c r="B2" s="56" t="s">
+        <v>128</v>
+      </c>
+      <c r="C2" s="56"/>
+      <c r="E2" s="52" t="s">
+        <v>221</v>
+      </c>
+      <c r="F2" s="52"/>
+      <c r="H2" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="I2" s="52"/>
+      <c r="K2" s="52" t="s">
         <v>223</v>
       </c>
-      <c r="F2" s="57"/>
-      <c r="H2" s="57" t="s">
+      <c r="L2" s="52"/>
+      <c r="N2" s="52" t="s">
         <v>224</v>
       </c>
-      <c r="I2" s="57"/>
-      <c r="K2" s="57" t="s">
+      <c r="O2" s="52"/>
+      <c r="Q2" s="52" t="s">
         <v>225</v>
       </c>
-      <c r="L2" s="57"/>
-      <c r="N2" s="57" t="s">
-        <v>226</v>
-      </c>
-      <c r="O2" s="57"/>
-      <c r="Q2" s="57" t="s">
-        <v>227</v>
-      </c>
-      <c r="R2" s="57"/>
+      <c r="R2" s="52"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="E3" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="F3" s="39"/>
-      <c r="H3" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="I3" s="39"/>
-      <c r="K3" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="L3" s="39"/>
-      <c r="N3" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="O3" s="39"/>
-      <c r="Q3" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="R3" s="39"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="E3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="35"/>
+      <c r="H3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="I3" s="35"/>
+      <c r="K3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="L3" s="35"/>
+      <c r="N3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="O3" s="35"/>
+      <c r="Q3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="R3" s="35"/>
       <c r="T3" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="28" t="s">
+      <c r="E4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="28" t="s">
+      <c r="H4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="28" t="s">
+      <c r="I4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="28" t="s">
+      <c r="K4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="L4" s="28" t="s">
+      <c r="L4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="28" t="s">
+      <c r="N4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="O4" s="28" t="s">
+      <c r="O4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="Q4" s="28" t="s">
+      <c r="Q4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="R4" s="28" t="s">
+      <c r="R4" s="25" t="s">
         <v>4</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="U4" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -12906,10 +12930,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="U5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -13208,318 +13232,301 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A900FC-A692-B445-95C9-59E70352B291}">
-  <dimension ref="A2:AK51"/>
+  <dimension ref="A2:AL52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
     <col min="3" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="35" width="8.5" customWidth="1"/>
-    <col min="36" max="36" width="8.5" style="1" customWidth="1"/>
-    <col min="37" max="37" width="8.5" customWidth="1"/>
+    <col min="11" max="38" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:38" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E2"/>
       <c r="F2"/>
       <c r="G2"/>
-      <c r="K2" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="Y2" s="6"/>
-      <c r="AE2" s="6" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="L2" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="AB2" s="6"/>
+      <c r="AH2" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:38" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F3"/>
       <c r="G3"/>
-      <c r="K3" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="L3" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y3" s="14"/>
-      <c r="AE3" s="1" t="s">
+      <c r="O3" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="P3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB3" s="14"/>
+      <c r="AH3" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="AI3" t="s">
         <v>168</v>
       </c>
-      <c r="AF3" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:38" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" t="s">
         <v>70</v>
-      </c>
-      <c r="D4" t="s">
-        <v>71</v>
       </c>
       <c r="F4"/>
       <c r="G4"/>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="42"/>
+      <c r="M4" t="s">
+        <v>161</v>
+      </c>
+      <c r="O4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="L4" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y4" s="14"/>
-      <c r="AE4" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="AF4" t="s">
+      <c r="P4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB4" s="14"/>
+      <c r="AH4" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="C5" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="D5" t="s">
+        <v>191</v>
+      </c>
+      <c r="L5" s="26"/>
+      <c r="M5" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="P5" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB5" s="14"/>
+      <c r="AH5" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="AI5" s="9" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="6" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="C6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="L6" s="29"/>
+      <c r="M6" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="P6" t="s">
+        <v>190</v>
+      </c>
+      <c r="AC6" s="1"/>
+      <c r="AD6" s="1"/>
+    </row>
+    <row r="7" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="C7" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="AC7" s="1"/>
+      <c r="AD7" s="1"/>
+    </row>
+    <row r="9" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="C9" s="45" t="s">
+        <v>236</v>
+      </c>
+      <c r="D9" s="45"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="45"/>
+      <c r="I9" s="45"/>
+      <c r="J9" s="45"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="45"/>
+      <c r="M9" s="45"/>
+      <c r="N9" s="45"/>
+      <c r="O9" s="45"/>
+      <c r="P9" s="45"/>
+      <c r="Q9" s="45"/>
+      <c r="R9" s="45"/>
+      <c r="S9" s="45"/>
+      <c r="T9" s="45"/>
+      <c r="U9" s="45"/>
+      <c r="V9" s="45"/>
+      <c r="W9" s="45"/>
+      <c r="X9" s="45"/>
+      <c r="Y9" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z9" s="45"/>
+      <c r="AA9" s="45"/>
+      <c r="AB9" s="45"/>
+      <c r="AC9" s="45"/>
+      <c r="AD9" s="45"/>
+      <c r="AE9" s="45" t="s">
+        <v>91</v>
+      </c>
+      <c r="AF9" s="45"/>
+      <c r="AG9" s="45"/>
+      <c r="AH9" s="45"/>
+      <c r="AI9" s="45"/>
+      <c r="AJ9" s="45"/>
+      <c r="AK9" s="45"/>
+      <c r="AL9" s="45"/>
+    </row>
+    <row r="10" spans="1:38" ht="18" x14ac:dyDescent="0.25">
+      <c r="A10" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="58" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="62" t="s">
+        <v>189</v>
+      </c>
+      <c r="E10" s="57" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="57" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" s="57" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" s="57" t="s">
+        <v>71</v>
+      </c>
+      <c r="J10" s="64" t="s">
+        <v>79</v>
+      </c>
+      <c r="K10" s="64" t="s">
+        <v>135</v>
+      </c>
+      <c r="L10" s="63" t="s">
+        <v>235</v>
+      </c>
+      <c r="M10" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="N10" s="43" t="s">
+        <v>211</v>
+      </c>
+      <c r="O10" s="57" t="s">
+        <v>84</v>
+      </c>
+      <c r="P10" s="57" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q10" s="57" t="s">
+        <v>173</v>
+      </c>
+      <c r="R10" s="57" t="s">
+        <v>174</v>
+      </c>
+      <c r="S10" s="57" t="s">
+        <v>175</v>
+      </c>
+      <c r="T10" s="57" t="s">
+        <v>176</v>
+      </c>
+      <c r="U10" s="57" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="C5" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D5" t="s">
-        <v>193</v>
-      </c>
-      <c r="K5" s="1" t="s">
+      <c r="V10" s="57" t="s">
+        <v>208</v>
+      </c>
+      <c r="W10" s="57" t="s">
+        <v>209</v>
+      </c>
+      <c r="X10" s="57" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y10" s="59" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z10" s="59" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA10" s="60" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB10" s="59" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC10" s="59" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD10" s="60" t="s">
+        <v>136</v>
+      </c>
+      <c r="AE10" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="L5" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="Y5" s="14"/>
-      <c r="AE5" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="AF5" s="9" t="s">
+      <c r="AF10" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="AG10" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="AH10" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="AI10" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="AJ10" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK10" s="23" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="C6" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>209</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="L6" t="s">
-        <v>192</v>
-      </c>
-      <c r="T6" s="1"/>
-      <c r="Z6" s="1"/>
-      <c r="AA6" s="1"/>
-    </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="C8" s="50" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" s="50"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="50"/>
-      <c r="G8" s="50"/>
-      <c r="H8" s="50"/>
-      <c r="I8" s="50"/>
-      <c r="J8" s="50"/>
-      <c r="K8" s="50"/>
-      <c r="L8" s="50"/>
-      <c r="M8" s="50"/>
-      <c r="N8" s="50"/>
-      <c r="O8" s="50"/>
-      <c r="P8" s="50"/>
-      <c r="Q8" s="50"/>
-      <c r="R8" s="50"/>
-      <c r="S8" s="50"/>
-      <c r="T8" s="50"/>
-      <c r="U8" s="50"/>
-      <c r="V8" s="50" t="s">
-        <v>58</v>
-      </c>
-      <c r="W8" s="50"/>
-      <c r="X8" s="50"/>
-      <c r="Y8" s="50"/>
-      <c r="Z8" s="50"/>
-      <c r="AA8" s="50"/>
-      <c r="AB8" s="50" t="s">
-        <v>92</v>
-      </c>
-      <c r="AC8" s="50"/>
-      <c r="AD8" s="50"/>
-      <c r="AE8" s="50"/>
-      <c r="AF8" s="50"/>
-      <c r="AG8" s="50"/>
-      <c r="AH8" s="50"/>
-      <c r="AI8" s="50"/>
-      <c r="AJ8" s="50" t="s">
+      <c r="AL10" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="AK8" s="50"/>
-    </row>
-    <row r="9" spans="1:37" ht="18" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="47" t="s">
-        <v>191</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="F9" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="H9" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="I9" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="J9" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="K9" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="L9" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="M9" s="21" t="s">
-        <v>176</v>
-      </c>
-      <c r="N9" s="21" t="s">
-        <v>177</v>
-      </c>
-      <c r="O9" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="P9" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="Q9" s="21" t="s">
-        <v>210</v>
-      </c>
-      <c r="R9" s="21" t="s">
-        <v>211</v>
-      </c>
-      <c r="S9" s="21" t="s">
-        <v>212</v>
-      </c>
-      <c r="T9" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="U9" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="V9" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="W9" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="X9" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="Y9" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="Z9" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA9" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="AB9" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="AC9" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="AD9" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="AE9" s="25" t="s">
-        <v>167</v>
-      </c>
-      <c r="AF9" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="AG9" s="25" t="s">
-        <v>96</v>
-      </c>
-      <c r="AH9" s="25" t="s">
-        <v>207</v>
-      </c>
-      <c r="AI9" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="AJ9" s="29" t="s">
-        <v>99</v>
-      </c>
-      <c r="AK9" s="48" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
+    </row>
+    <row r="11" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
         <v>1</v>
-      </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="3"/>
-      <c r="T10" s="3"/>
-      <c r="U10" s="3"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
-      <c r="X10" s="3"/>
-      <c r="Y10" s="3"/>
-      <c r="Z10" s="3"/>
-      <c r="AA10" s="3"/>
-      <c r="AB10" s="3"/>
-      <c r="AC10" s="3"/>
-      <c r="AD10" s="3"/>
-      <c r="AE10" s="3"/>
-      <c r="AF10" s="3"/>
-      <c r="AG10" s="3"/>
-      <c r="AH10" s="3"/>
-      <c r="AI10" s="3"/>
-      <c r="AJ10" s="3"/>
-      <c r="AK10" s="3"/>
-    </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
-        <v>2</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -13553,14 +13560,15 @@
       <c r="AE11" s="3"/>
       <c r="AF11" s="3"/>
       <c r="AG11" s="3"/>
-      <c r="AH11" s="18"/>
-      <c r="AI11" s="19"/>
+      <c r="AH11" s="3"/>
+      <c r="AI11" s="3"/>
       <c r="AJ11" s="3"/>
       <c r="AK11" s="3"/>
-    </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL11" s="3"/>
+    </row>
+    <row r="12" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -13594,14 +13602,15 @@
       <c r="AE12" s="3"/>
       <c r="AF12" s="3"/>
       <c r="AG12" s="3"/>
-      <c r="AH12" s="18"/>
-      <c r="AI12" s="19"/>
+      <c r="AH12" s="3"/>
+      <c r="AI12" s="3"/>
       <c r="AJ12" s="3"/>
-      <c r="AK12" s="3"/>
-    </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AK12" s="18"/>
+      <c r="AL12" s="19"/>
+    </row>
+    <row r="13" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -13638,11 +13647,12 @@
       <c r="AH13" s="3"/>
       <c r="AI13" s="3"/>
       <c r="AJ13" s="3"/>
-      <c r="AK13" s="3"/>
-    </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AK13" s="18"/>
+      <c r="AL13" s="19"/>
+    </row>
+    <row r="14" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -13680,10 +13690,11 @@
       <c r="AI14" s="3"/>
       <c r="AJ14" s="3"/>
       <c r="AK14" s="3"/>
-    </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL14" s="3"/>
+    </row>
+    <row r="15" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -13721,10 +13732,11 @@
       <c r="AI15" s="3"/>
       <c r="AJ15" s="3"/>
       <c r="AK15" s="3"/>
-    </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL15" s="3"/>
+    </row>
+    <row r="16" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -13762,10 +13774,11 @@
       <c r="AI16" s="3"/>
       <c r="AJ16" s="3"/>
       <c r="AK16" s="3"/>
-    </row>
-    <row r="17" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL16" s="3"/>
+    </row>
+    <row r="17" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -13803,10 +13816,11 @@
       <c r="AI17" s="3"/>
       <c r="AJ17" s="3"/>
       <c r="AK17" s="3"/>
-    </row>
-    <row r="18" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL17" s="3"/>
+    </row>
+    <row r="18" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -13844,10 +13858,11 @@
       <c r="AI18" s="3"/>
       <c r="AJ18" s="3"/>
       <c r="AK18" s="3"/>
-    </row>
-    <row r="19" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL18" s="3"/>
+    </row>
+    <row r="19" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -13885,10 +13900,11 @@
       <c r="AI19" s="3"/>
       <c r="AJ19" s="3"/>
       <c r="AK19" s="3"/>
-    </row>
-    <row r="20" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL19" s="3"/>
+    </row>
+    <row r="20" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -13926,10 +13942,11 @@
       <c r="AI20" s="3"/>
       <c r="AJ20" s="3"/>
       <c r="AK20" s="3"/>
-    </row>
-    <row r="21" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL20" s="3"/>
+    </row>
+    <row r="21" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -13967,10 +13984,11 @@
       <c r="AI21" s="3"/>
       <c r="AJ21" s="3"/>
       <c r="AK21" s="3"/>
-    </row>
-    <row r="22" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL21" s="3"/>
+    </row>
+    <row r="22" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -14008,10 +14026,11 @@
       <c r="AI22" s="3"/>
       <c r="AJ22" s="3"/>
       <c r="AK22" s="3"/>
-    </row>
-    <row r="23" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL22" s="3"/>
+    </row>
+    <row r="23" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -14049,10 +14068,11 @@
       <c r="AI23" s="3"/>
       <c r="AJ23" s="3"/>
       <c r="AK23" s="3"/>
-    </row>
-    <row r="24" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL23" s="3"/>
+    </row>
+    <row r="24" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -14090,35 +14110,51 @@
       <c r="AI24" s="3"/>
       <c r="AJ24" s="3"/>
       <c r="AK24" s="3"/>
-    </row>
-    <row r="25" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="K25" s="1"/>
-      <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
-      <c r="N25" s="1"/>
-      <c r="O25" s="1"/>
-      <c r="P25" s="1"/>
-      <c r="Q25" s="1"/>
-      <c r="R25" s="1"/>
-      <c r="S25" s="1"/>
-      <c r="T25" s="1"/>
-      <c r="U25" s="1"/>
-      <c r="V25" s="1"/>
-      <c r="W25" s="1"/>
-      <c r="X25" s="1"/>
-      <c r="Y25" s="1"/>
-      <c r="Z25" s="1"/>
-      <c r="AA25" s="1"/>
-      <c r="AB25" s="1"/>
-      <c r="AC25" s="1"/>
-      <c r="AD25" s="1"/>
-      <c r="AE25" s="1"/>
-      <c r="AF25" s="1"/>
-      <c r="AG25" s="1"/>
-      <c r="AH25" s="1"/>
-      <c r="AI25" s="1"/>
-    </row>
-    <row r="26" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL24" s="3"/>
+    </row>
+    <row r="25" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>15</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="3"/>
+      <c r="V25" s="3"/>
+      <c r="W25" s="3"/>
+      <c r="X25" s="3"/>
+      <c r="Y25" s="3"/>
+      <c r="Z25" s="3"/>
+      <c r="AA25" s="3"/>
+      <c r="AB25" s="3"/>
+      <c r="AC25" s="3"/>
+      <c r="AD25" s="3"/>
+      <c r="AE25" s="3"/>
+      <c r="AF25" s="3"/>
+      <c r="AG25" s="3"/>
+      <c r="AH25" s="3"/>
+      <c r="AI25" s="3"/>
+      <c r="AJ25" s="3"/>
+      <c r="AK25" s="3"/>
+      <c r="AL25" s="3"/>
+    </row>
+    <row r="26" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -14136,8 +14172,19 @@
       <c r="Y26" s="1"/>
       <c r="Z26" s="1"/>
       <c r="AA26" s="1"/>
-    </row>
-    <row r="27" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB26" s="1"/>
+      <c r="AC26" s="1"/>
+      <c r="AD26" s="1"/>
+      <c r="AE26" s="1"/>
+      <c r="AF26" s="1"/>
+      <c r="AG26" s="1"/>
+      <c r="AH26" s="1"/>
+      <c r="AI26" s="1"/>
+      <c r="AJ26" s="1"/>
+      <c r="AK26" s="1"/>
+      <c r="AL26" s="1"/>
+    </row>
+    <row r="27" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -14155,8 +14202,11 @@
       <c r="Y27" s="1"/>
       <c r="Z27" s="1"/>
       <c r="AA27" s="1"/>
-    </row>
-    <row r="28" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB27" s="1"/>
+      <c r="AC27" s="1"/>
+      <c r="AD27" s="1"/>
+    </row>
+    <row r="28" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -14174,8 +14224,11 @@
       <c r="Y28" s="1"/>
       <c r="Z28" s="1"/>
       <c r="AA28" s="1"/>
-    </row>
-    <row r="29" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB28" s="1"/>
+      <c r="AC28" s="1"/>
+      <c r="AD28" s="1"/>
+    </row>
+    <row r="29" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -14193,8 +14246,11 @@
       <c r="Y29" s="1"/>
       <c r="Z29" s="1"/>
       <c r="AA29" s="1"/>
-    </row>
-    <row r="30" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB29" s="1"/>
+      <c r="AC29" s="1"/>
+      <c r="AD29" s="1"/>
+    </row>
+    <row r="30" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -14212,8 +14268,11 @@
       <c r="Y30" s="1"/>
       <c r="Z30" s="1"/>
       <c r="AA30" s="1"/>
-    </row>
-    <row r="31" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB30" s="1"/>
+      <c r="AC30" s="1"/>
+      <c r="AD30" s="1"/>
+    </row>
+    <row r="31" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -14231,8 +14290,11 @@
       <c r="Y31" s="1"/>
       <c r="Z31" s="1"/>
       <c r="AA31" s="1"/>
-    </row>
-    <row r="32" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB31" s="1"/>
+      <c r="AC31" s="1"/>
+      <c r="AD31" s="1"/>
+    </row>
+    <row r="32" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -14250,8 +14312,11 @@
       <c r="Y32" s="1"/>
       <c r="Z32" s="1"/>
       <c r="AA32" s="1"/>
-    </row>
-    <row r="33" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB32" s="1"/>
+      <c r="AC32" s="1"/>
+      <c r="AD32" s="1"/>
+    </row>
+    <row r="33" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
@@ -14269,8 +14334,11 @@
       <c r="Y33" s="1"/>
       <c r="Z33" s="1"/>
       <c r="AA33" s="1"/>
-    </row>
-    <row r="34" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB33" s="1"/>
+      <c r="AC33" s="1"/>
+      <c r="AD33" s="1"/>
+    </row>
+    <row r="34" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
@@ -14288,8 +14356,11 @@
       <c r="Y34" s="1"/>
       <c r="Z34" s="1"/>
       <c r="AA34" s="1"/>
-    </row>
-    <row r="35" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB34" s="1"/>
+      <c r="AC34" s="1"/>
+      <c r="AD34" s="1"/>
+    </row>
+    <row r="35" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
@@ -14307,8 +14378,11 @@
       <c r="Y35" s="1"/>
       <c r="Z35" s="1"/>
       <c r="AA35" s="1"/>
-    </row>
-    <row r="36" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB35" s="1"/>
+      <c r="AC35" s="1"/>
+      <c r="AD35" s="1"/>
+    </row>
+    <row r="36" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -14326,8 +14400,11 @@
       <c r="Y36" s="1"/>
       <c r="Z36" s="1"/>
       <c r="AA36" s="1"/>
-    </row>
-    <row r="37" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB36" s="1"/>
+      <c r="AC36" s="1"/>
+      <c r="AD36" s="1"/>
+    </row>
+    <row r="37" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
@@ -14345,8 +14422,11 @@
       <c r="Y37" s="1"/>
       <c r="Z37" s="1"/>
       <c r="AA37" s="1"/>
-    </row>
-    <row r="38" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB37" s="1"/>
+      <c r="AC37" s="1"/>
+      <c r="AD37" s="1"/>
+    </row>
+    <row r="38" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
@@ -14364,8 +14444,11 @@
       <c r="Y38" s="1"/>
       <c r="Z38" s="1"/>
       <c r="AA38" s="1"/>
-    </row>
-    <row r="39" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB38" s="1"/>
+      <c r="AC38" s="1"/>
+      <c r="AD38" s="1"/>
+    </row>
+    <row r="39" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -14383,8 +14466,11 @@
       <c r="Y39" s="1"/>
       <c r="Z39" s="1"/>
       <c r="AA39" s="1"/>
-    </row>
-    <row r="40" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB39" s="1"/>
+      <c r="AC39" s="1"/>
+      <c r="AD39" s="1"/>
+    </row>
+    <row r="40" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
@@ -14402,8 +14488,11 @@
       <c r="Y40" s="1"/>
       <c r="Z40" s="1"/>
       <c r="AA40" s="1"/>
-    </row>
-    <row r="41" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB40" s="1"/>
+      <c r="AC40" s="1"/>
+      <c r="AD40" s="1"/>
+    </row>
+    <row r="41" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
@@ -14421,8 +14510,11 @@
       <c r="Y41" s="1"/>
       <c r="Z41" s="1"/>
       <c r="AA41" s="1"/>
-    </row>
-    <row r="42" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB41" s="1"/>
+      <c r="AC41" s="1"/>
+      <c r="AD41" s="1"/>
+    </row>
+    <row r="42" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
@@ -14440,8 +14532,11 @@
       <c r="Y42" s="1"/>
       <c r="Z42" s="1"/>
       <c r="AA42" s="1"/>
-    </row>
-    <row r="43" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB42" s="1"/>
+      <c r="AC42" s="1"/>
+      <c r="AD42" s="1"/>
+    </row>
+    <row r="43" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
@@ -14459,8 +14554,11 @@
       <c r="Y43" s="1"/>
       <c r="Z43" s="1"/>
       <c r="AA43" s="1"/>
-    </row>
-    <row r="44" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB43" s="1"/>
+      <c r="AC43" s="1"/>
+      <c r="AD43" s="1"/>
+    </row>
+    <row r="44" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
@@ -14478,8 +14576,11 @@
       <c r="Y44" s="1"/>
       <c r="Z44" s="1"/>
       <c r="AA44" s="1"/>
-    </row>
-    <row r="45" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB44" s="1"/>
+      <c r="AC44" s="1"/>
+      <c r="AD44" s="1"/>
+    </row>
+    <row r="45" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
@@ -14497,8 +14598,11 @@
       <c r="Y45" s="1"/>
       <c r="Z45" s="1"/>
       <c r="AA45" s="1"/>
-    </row>
-    <row r="46" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB45" s="1"/>
+      <c r="AC45" s="1"/>
+      <c r="AD45" s="1"/>
+    </row>
+    <row r="46" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
@@ -14516,8 +14620,11 @@
       <c r="Y46" s="1"/>
       <c r="Z46" s="1"/>
       <c r="AA46" s="1"/>
-    </row>
-    <row r="47" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB46" s="1"/>
+      <c r="AC46" s="1"/>
+      <c r="AD46" s="1"/>
+    </row>
+    <row r="47" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
       <c r="M47" s="1"/>
@@ -14535,8 +14642,11 @@
       <c r="Y47" s="1"/>
       <c r="Z47" s="1"/>
       <c r="AA47" s="1"/>
-    </row>
-    <row r="48" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB47" s="1"/>
+      <c r="AC47" s="1"/>
+      <c r="AD47" s="1"/>
+    </row>
+    <row r="48" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
@@ -14554,8 +14664,11 @@
       <c r="Y48" s="1"/>
       <c r="Z48" s="1"/>
       <c r="AA48" s="1"/>
-    </row>
-    <row r="49" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB48" s="1"/>
+      <c r="AC48" s="1"/>
+      <c r="AD48" s="1"/>
+    </row>
+    <row r="49" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
@@ -14573,8 +14686,11 @@
       <c r="Y49" s="1"/>
       <c r="Z49" s="1"/>
       <c r="AA49" s="1"/>
-    </row>
-    <row r="50" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB49" s="1"/>
+      <c r="AC49" s="1"/>
+      <c r="AD49" s="1"/>
+    </row>
+    <row r="50" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K50" s="1"/>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
@@ -14592,8 +14708,11 @@
       <c r="Y50" s="1"/>
       <c r="Z50" s="1"/>
       <c r="AA50" s="1"/>
-    </row>
-    <row r="51" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB50" s="1"/>
+      <c r="AC50" s="1"/>
+      <c r="AD50" s="1"/>
+    </row>
+    <row r="51" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
@@ -14611,88 +14730,125 @@
       <c r="Y51" s="1"/>
       <c r="Z51" s="1"/>
       <c r="AA51" s="1"/>
+      <c r="AB51" s="1"/>
+      <c r="AC51" s="1"/>
+      <c r="AD51" s="1"/>
+    </row>
+    <row r="52" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="K52" s="1"/>
+      <c r="L52" s="1"/>
+      <c r="M52" s="1"/>
+      <c r="N52" s="1"/>
+      <c r="O52" s="1"/>
+      <c r="P52" s="1"/>
+      <c r="Q52" s="1"/>
+      <c r="R52" s="1"/>
+      <c r="S52" s="1"/>
+      <c r="T52" s="1"/>
+      <c r="U52" s="1"/>
+      <c r="V52" s="1"/>
+      <c r="W52" s="1"/>
+      <c r="X52" s="1"/>
+      <c r="Y52" s="1"/>
+      <c r="Z52" s="1"/>
+      <c r="AA52" s="1"/>
+      <c r="AB52" s="1"/>
+      <c r="AC52" s="1"/>
+      <c r="AD52" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="V8:AA8"/>
-    <mergeCell ref="AJ8:AK8"/>
-    <mergeCell ref="AB8:AI8"/>
-    <mergeCell ref="C8:U8"/>
+  <mergeCells count="3">
+    <mergeCell ref="Y9:AD9"/>
+    <mergeCell ref="AE9:AL9"/>
+    <mergeCell ref="C9:X9"/>
   </mergeCells>
-  <conditionalFormatting sqref="F10:K51 W10:AA51">
-    <cfRule type="expression" dxfId="15" priority="2">
-      <formula>$E10="hb"</formula>
+  <conditionalFormatting sqref="F11:K52 Z11:AD52">
+    <cfRule type="expression" dxfId="5" priority="1">
+      <formula>$E11="hb"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="2">
+      <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G10:G51">
-    <cfRule type="expression" dxfId="14" priority="7">
-      <formula>$E10="cp"</formula>
+  <conditionalFormatting sqref="G11:G52">
+    <cfRule type="expression" dxfId="5" priority="3">
+      <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H10:I51">
-    <cfRule type="expression" dxfId="13" priority="6">
-      <formula>$E10="mc"</formula>
+  <conditionalFormatting sqref="H11:I52">
+    <cfRule type="expression" dxfId="5" priority="4">
+      <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J10:K51">
-    <cfRule type="expression" dxfId="12" priority="8">
-      <formula>$E10="cp"</formula>
+  <conditionalFormatting sqref="J11:K52">
+    <cfRule type="expression" dxfId="5" priority="5">
+      <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L10:O51">
-    <cfRule type="expression" dxfId="11" priority="21">
-      <formula>AND($E10&lt;&gt;"",$E10&lt;&gt;"pow")</formula>
+  <conditionalFormatting sqref="Q11:T52">
+    <cfRule type="expression" dxfId="5" priority="6">
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P10:S51">
-    <cfRule type="expression" dxfId="10" priority="1">
-      <formula>AND($E10&lt;&gt;"",$E10&lt;&gt;"hb")</formula>
+  <conditionalFormatting sqref="U11:X52">
+    <cfRule type="expression" dxfId="5" priority="7">
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U10:U51">
-    <cfRule type="expression" dxfId="9" priority="22">
-      <formula>AND($T10&lt;&gt;"",$T10&lt;&gt;"ru")</formula>
+  <conditionalFormatting sqref="P11:P52">
+    <cfRule type="expression" dxfId="5" priority="8">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W10:AA51 F10:K51">
-    <cfRule type="expression" dxfId="8" priority="18">
-      <formula>$E10="pow"</formula>
+  <conditionalFormatting sqref="AA11:AA52">
+    <cfRule type="expression" dxfId="5" priority="9">
+      <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X10:X51">
-    <cfRule type="expression" dxfId="7" priority="10">
-      <formula>$E10="cp"</formula>
+  <conditionalFormatting sqref="AB11:AB52">
+    <cfRule type="expression" dxfId="5" priority="10">
+      <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y10:Y51">
-    <cfRule type="expression" dxfId="6" priority="17">
-      <formula>$E10="mc"</formula>
+  <conditionalFormatting sqref="AC11:AD52">
+    <cfRule type="expression" dxfId="5" priority="11">
+      <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z10:AA51">
+  <conditionalFormatting sqref="AI11:AJ52">
     <cfRule type="expression" dxfId="5" priority="12">
-      <formula>$E10="cp"</formula>
+      <formula>OR($AH11="vg",$AH11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AF10:AG101">
-    <cfRule type="expression" dxfId="4" priority="4">
-      <formula>OR($AE10="vg",$AE10="gard")</formula>
+  <conditionalFormatting sqref="AK11:AL52">
+    <cfRule type="expression" dxfId="5" priority="13">
+      <formula>$AH11="lf"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AH10:AI101">
-    <cfRule type="expression" dxfId="3" priority="3">
-      <formula>$AE10="lf"</formula>
+  <conditionalFormatting sqref="F11:L52">
+    <cfRule type="expression" dxfId="5" priority="14">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O11:P52">
+    <cfRule type="expression" dxfId="5" priority="15">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z11:AD52">
+    <cfRule type="expression" dxfId="5" priority="16">
+      <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E10:E51" xr:uid="{374AFD2C-B540-DD4B-A245-8B781F76E64C}">
-      <formula1>$C$3:$C$6</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11:E52" xr:uid="{374AFD2C-B540-DD4B-A245-8B781F76E64C}">
+      <formula1>$C$3:$C$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T10:T51" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
-      <formula1>$K$3:$K$6</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH11:AH102" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
+      <formula1>$AH$3:$AH$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE10:AE101" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
-      <formula1>$AE$3:$AE$5</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O11:O52" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
+      <formula1>$O$3:$O$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14732,264 +14888,264 @@
       <c r="B2" s="3">
         <v>0</v>
       </c>
-      <c r="D2" s="27" t="s">
-        <v>93</v>
+      <c r="D2" s="24" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="D4" s="51" t="s">
+      <c r="B4" s="48"/>
+      <c r="D4" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="51"/>
-      <c r="G4" s="51" t="s">
+      <c r="E4" s="48"/>
+      <c r="G4" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="51"/>
-      <c r="J4" s="51" t="s">
+      <c r="H4" s="48"/>
+      <c r="J4" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="51"/>
-      <c r="M4" s="51" t="s">
+      <c r="K4" s="48"/>
+      <c r="M4" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="51"/>
-      <c r="P4" s="51" t="s">
+      <c r="N4" s="48"/>
+      <c r="P4" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="51"/>
+      <c r="Q4" s="48"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="51" t="s">
+      <c r="S4" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="51"/>
+      <c r="T4" s="48"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="51" t="s">
+      <c r="V4" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="51"/>
+      <c r="W4" s="48"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="51" t="s">
+      <c r="Y4" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="51"/>
+      <c r="Z4" s="48"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="51" t="s">
+      <c r="AB4" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="51"/>
-      <c r="AE4" s="51" t="s">
+      <c r="AC4" s="48"/>
+      <c r="AE4" s="48" t="s">
+        <v>108</v>
+      </c>
+      <c r="AF4" s="48"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="48" t="s">
+        <v>109</v>
+      </c>
+      <c r="AI4" s="48"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="48" t="s">
         <v>110</v>
       </c>
-      <c r="AF4" s="51"/>
-      <c r="AG4" s="1"/>
-      <c r="AH4" s="51" t="s">
+      <c r="AL4" s="48"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="48" t="s">
         <v>111</v>
       </c>
-      <c r="AI4" s="51"/>
-      <c r="AJ4" s="1"/>
-      <c r="AK4" s="51" t="s">
+      <c r="AO4" s="48"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="AL4" s="51"/>
-      <c r="AM4" s="1"/>
-      <c r="AN4" s="51" t="s">
-        <v>113</v>
-      </c>
-      <c r="AO4" s="51"/>
-      <c r="AP4" s="1"/>
-      <c r="AQ4" s="51" t="s">
-        <v>114</v>
-      </c>
-      <c r="AR4" s="51"/>
+      <c r="AR4" s="48"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="B5" s="41">
+      <c r="A5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="37">
         <v>1</v>
       </c>
-      <c r="D5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="E5" s="41">
+      <c r="D5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" s="37">
         <v>2</v>
       </c>
-      <c r="G5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="H5" s="41">
+      <c r="G5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="H5" s="37">
         <v>3</v>
       </c>
-      <c r="J5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="K5" s="41">
+      <c r="J5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="K5" s="37">
         <v>4</v>
       </c>
-      <c r="M5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="N5" s="41">
+      <c r="M5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="N5" s="37">
         <v>5</v>
       </c>
-      <c r="P5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q5" s="41">
+      <c r="P5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q5" s="37">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
-      <c r="S5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="T5" s="41">
+      <c r="S5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="T5" s="37">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
-      <c r="V5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="W5" s="41">
+      <c r="V5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="W5" s="37">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
-      <c r="Y5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="Z5" s="41">
+      <c r="Y5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z5" s="37">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
-      <c r="AB5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AC5" s="41">
+      <c r="AB5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AC5" s="37">
         <v>10</v>
       </c>
-      <c r="AE5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AF5" s="41">
+      <c r="AE5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF5" s="37">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
-      <c r="AH5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AI5" s="41">
+      <c r="AH5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AI5" s="37">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
-      <c r="AK5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AL5" s="41">
+      <c r="AK5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AL5" s="37">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
-      <c r="AN5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AO5" s="41">
+      <c r="AN5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AO5" s="37">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
-      <c r="AQ5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AR5" s="41">
+      <c r="AQ5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AR5" s="37">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="52" t="str">
+      <c r="A6" s="46" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="53"/>
-      <c r="D6" s="52" t="str">
+      <c r="B6" s="47"/>
+      <c r="D6" s="46" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="53"/>
-      <c r="G6" s="52" t="str">
+      <c r="E6" s="47"/>
+      <c r="G6" s="46" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="53"/>
-      <c r="J6" s="52" t="str">
+      <c r="H6" s="47"/>
+      <c r="J6" s="46" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="53"/>
-      <c r="M6" s="52" t="str">
+      <c r="K6" s="47"/>
+      <c r="M6" s="46" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="53"/>
-      <c r="P6" s="52" t="str">
+      <c r="N6" s="47"/>
+      <c r="P6" s="46" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="53"/>
+      <c r="Q6" s="47"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="52" t="str">
+      <c r="S6" s="46" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="53"/>
+      <c r="T6" s="47"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="52" t="str">
+      <c r="V6" s="46" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="53"/>
+      <c r="W6" s="47"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="52" t="str">
+      <c r="Y6" s="46" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="53"/>
+      <c r="Z6" s="47"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="52" t="str">
+      <c r="AB6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="53"/>
-      <c r="AE6" s="52" t="str">
+      <c r="AC6" s="47"/>
+      <c r="AE6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="53"/>
+      <c r="AF6" s="47"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="52" t="str">
+      <c r="AH6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="53"/>
+      <c r="AI6" s="47"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="52" t="str">
+      <c r="AK6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="53"/>
+      <c r="AL6" s="47"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="52" t="str">
+      <c r="AN6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="53"/>
+      <c r="AO6" s="47"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="52" t="str">
+      <c r="AQ6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="53"/>
+      <c r="AR6" s="47"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -15893,36 +16049,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15955,264 +16111,264 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A2" s="27" t="s">
-        <v>158</v>
+      <c r="A2" s="24" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="48"/>
+      <c r="D4" s="48" t="s">
+        <v>138</v>
+      </c>
+      <c r="E4" s="48"/>
+      <c r="G4" s="48" t="s">
         <v>139</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="D4" s="51" t="s">
+      <c r="H4" s="48"/>
+      <c r="J4" s="48" t="s">
         <v>140</v>
       </c>
-      <c r="E4" s="51"/>
-      <c r="G4" s="51" t="s">
+      <c r="K4" s="48"/>
+      <c r="M4" s="48" t="s">
         <v>141</v>
       </c>
-      <c r="H4" s="51"/>
-      <c r="J4" s="51" t="s">
+      <c r="N4" s="48"/>
+      <c r="P4" s="48" t="s">
         <v>142</v>
       </c>
-      <c r="K4" s="51"/>
-      <c r="M4" s="51" t="s">
+      <c r="Q4" s="48"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="48" t="s">
         <v>143</v>
       </c>
-      <c r="N4" s="51"/>
-      <c r="P4" s="51" t="s">
+      <c r="T4" s="48"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="48" t="s">
         <v>144</v>
       </c>
-      <c r="Q4" s="51"/>
-      <c r="R4" s="1"/>
-      <c r="S4" s="51" t="s">
+      <c r="W4" s="48"/>
+      <c r="X4" s="1"/>
+      <c r="Y4" s="48" t="s">
         <v>145</v>
       </c>
-      <c r="T4" s="51"/>
-      <c r="U4" s="1"/>
-      <c r="V4" s="51" t="s">
+      <c r="Z4" s="48"/>
+      <c r="AA4" s="1"/>
+      <c r="AB4" s="48" t="s">
         <v>146</v>
       </c>
-      <c r="W4" s="51"/>
-      <c r="X4" s="1"/>
-      <c r="Y4" s="51" t="s">
+      <c r="AC4" s="48"/>
+      <c r="AE4" s="48" t="s">
         <v>147</v>
       </c>
-      <c r="Z4" s="51"/>
-      <c r="AA4" s="1"/>
-      <c r="AB4" s="51" t="s">
+      <c r="AF4" s="48"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="AC4" s="51"/>
-      <c r="AE4" s="51" t="s">
+      <c r="AI4" s="48"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="48" t="s">
         <v>149</v>
       </c>
-      <c r="AF4" s="51"/>
-      <c r="AG4" s="1"/>
-      <c r="AH4" s="51" t="s">
+      <c r="AL4" s="48"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="48" t="s">
         <v>150</v>
       </c>
-      <c r="AI4" s="51"/>
-      <c r="AJ4" s="1"/>
-      <c r="AK4" s="51" t="s">
+      <c r="AO4" s="48"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="48" t="s">
         <v>151</v>
       </c>
-      <c r="AL4" s="51"/>
-      <c r="AM4" s="1"/>
-      <c r="AN4" s="51" t="s">
-        <v>152</v>
-      </c>
-      <c r="AO4" s="51"/>
-      <c r="AP4" s="1"/>
-      <c r="AQ4" s="51" t="s">
-        <v>153</v>
-      </c>
-      <c r="AR4" s="51"/>
+      <c r="AR4" s="48"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="B5" s="43">
+      <c r="A5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="39">
         <v>1</v>
       </c>
-      <c r="D5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="E5" s="43">
+      <c r="D5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" s="39">
         <v>2</v>
       </c>
-      <c r="G5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="H5" s="43">
+      <c r="G5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="H5" s="39">
         <v>3</v>
       </c>
-      <c r="J5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="K5" s="43">
+      <c r="J5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="K5" s="39">
         <v>4</v>
       </c>
-      <c r="M5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="N5" s="43">
+      <c r="M5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="N5" s="39">
         <v>5</v>
       </c>
-      <c r="P5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q5" s="43">
+      <c r="P5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q5" s="39">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
-      <c r="S5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="T5" s="43">
+      <c r="S5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="T5" s="39">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
-      <c r="V5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="W5" s="43">
+      <c r="V5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="W5" s="39">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
-      <c r="Y5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="Z5" s="43">
+      <c r="Y5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z5" s="39">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
-      <c r="AB5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AC5" s="43">
+      <c r="AB5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AC5" s="39">
         <v>10</v>
       </c>
-      <c r="AE5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AF5" s="43">
+      <c r="AE5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF5" s="39">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
-      <c r="AH5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AI5" s="43">
+      <c r="AH5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AI5" s="39">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
-      <c r="AK5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AL5" s="43">
+      <c r="AK5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AL5" s="39">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
-      <c r="AN5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AO5" s="43">
+      <c r="AN5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AO5" s="39">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
-      <c r="AQ5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AR5" s="43">
+      <c r="AQ5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AR5" s="39">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="54" t="str">
+      <c r="A6" s="49" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="55"/>
-      <c r="D6" s="54" t="str">
+      <c r="B6" s="50"/>
+      <c r="D6" s="49" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="55"/>
-      <c r="G6" s="54" t="str">
+      <c r="E6" s="50"/>
+      <c r="G6" s="49" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="55"/>
-      <c r="J6" s="54" t="str">
+      <c r="H6" s="50"/>
+      <c r="J6" s="49" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="55"/>
-      <c r="M6" s="54" t="str">
+      <c r="K6" s="50"/>
+      <c r="M6" s="49" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="55"/>
-      <c r="P6" s="54" t="str">
+      <c r="N6" s="50"/>
+      <c r="P6" s="49" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="55"/>
+      <c r="Q6" s="50"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="54" t="str">
+      <c r="S6" s="49" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="55"/>
+      <c r="T6" s="50"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="54" t="str">
+      <c r="V6" s="49" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="55"/>
+      <c r="W6" s="50"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="54" t="str">
+      <c r="Y6" s="49" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="55"/>
+      <c r="Z6" s="50"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="54" t="str">
+      <c r="AB6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="55"/>
-      <c r="AE6" s="54" t="str">
+      <c r="AC6" s="50"/>
+      <c r="AE6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="55"/>
+      <c r="AF6" s="50"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="54" t="str">
+      <c r="AH6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="55"/>
+      <c r="AI6" s="50"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="54" t="str">
+      <c r="AK6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="55"/>
+      <c r="AL6" s="50"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="54" t="str">
+      <c r="AN6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="55"/>
+      <c r="AO6" s="50"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="54" t="str">
+      <c r="AQ6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="55"/>
+      <c r="AR6" s="50"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -17116,14 +17272,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -17140,12 +17294,14 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17161,28 +17317,28 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="56"/>
-      <c r="D2" s="57" t="s">
+      <c r="A2" s="51" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="51"/>
+      <c r="D2" s="52" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" s="52"/>
+      <c r="G2" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="57"/>
-      <c r="G2" s="24" t="s">
-        <v>83</v>
-      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="36" t="s">
-        <v>198</v>
-      </c>
-      <c r="B3" s="37"/>
-      <c r="D3" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="E3" s="39"/>
-      <c r="G3" s="24"/>
+      <c r="A3" s="32" t="s">
+        <v>196</v>
+      </c>
+      <c r="B3" s="33"/>
+      <c r="D3" s="34" t="s">
+        <v>196</v>
+      </c>
+      <c r="E3" s="35"/>
+      <c r="G3" s="22"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
@@ -17198,7 +17354,7 @@
         <v>4</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H4" s="1"/>
     </row>
@@ -17211,7 +17367,7 @@
         <v>21</v>
       </c>
       <c r="H5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -17220,10 +17376,10 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="G6" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -17363,10 +17519,10 @@
         <v>25</v>
       </c>
       <c r="B2" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="13" t="s">
         <v>61</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>62</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>29</v>
@@ -17381,7 +17537,7 @@
         <v>28</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>30</v>
@@ -17438,10 +17594,10 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="J5" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -17613,10 +17769,10 @@
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" t="s">
+        <v>75</v>
+      </c>
+      <c r="F5" t="s">
         <v>76</v>
-      </c>
-      <c r="F5" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -17739,36 +17895,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="53" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="F2" s="53" t="s">
+        <v>122</v>
+      </c>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="J2" s="53" t="s">
         <v>123</v>
       </c>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="F2" s="58" t="s">
+      <c r="K2" s="53"/>
+      <c r="L2" s="53"/>
+      <c r="N2" s="53" t="s">
         <v>124</v>
       </c>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="J2" s="58" t="s">
+      <c r="O2" s="53"/>
+      <c r="P2" s="53"/>
+      <c r="R2" s="53" t="s">
         <v>125</v>
       </c>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="N2" s="58" t="s">
+      <c r="S2" s="53"/>
+      <c r="T2" s="53"/>
+      <c r="V2" s="53" t="s">
         <v>126</v>
       </c>
-      <c r="O2" s="58"/>
-      <c r="P2" s="58"/>
-      <c r="R2" s="58" t="s">
-        <v>127</v>
-      </c>
-      <c r="S2" s="58"/>
-      <c r="T2" s="58"/>
-      <c r="V2" s="58" t="s">
-        <v>128</v>
-      </c>
-      <c r="W2" s="58"/>
-      <c r="X2" s="58"/>
+      <c r="W2" s="53"/>
+      <c r="X2" s="53"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">

</xml_diff>

<commit_message>
chore(resources): ship v17 template; editor fixture carries phi_b/s_cap
xslope/resources/input_template.xlsx byte-synced to the v17 docs master (the copy
shipped in the wheel, used by the Studio assistant on pip installs) -- template_sync
guard green. The editor round-trip fixture's full material now sets the v17
phi_b/s_cap pair to distinct non-None values (None on the elastic row, mirroring
t_cut), so the editors' base-dict ride-along must preserve them through a build/apply
round-trip in both the table and list views.

save_slope_data_to_xlsx round-trips phi_b/s_cap via MAT_OPT_NUM_HEADERS: verified on
a 4-material file that None stays a blank cell, 0.0 is preserved as distinct from
blank, and per-material values survive independently.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/xslope/resources/input_template.xlsx
+++ b/xslope/resources/input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448736C4-E2C8-EB41-827A-888C500BCAB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9AE3CBE-0B2A-ED44-BB50-AACC6A5490D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="35040" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="240">
   <si>
     <t>X</t>
   </si>
@@ -941,6 +941,12 @@
   </si>
   <si>
     <t>Color legend</t>
+  </si>
+  <si>
+    <t>phi_b</t>
+  </si>
+  <si>
+    <t>s_cap</t>
   </si>
 </sst>
 </file>
@@ -1090,7 +1096,7 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1187,12 +1193,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="-0.499984740745262"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="7">
     <border>
@@ -1280,7 +1280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1397,19 +1397,37 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1436,35 +1454,11 @@
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="19">
     <dxf>
       <fill>
         <patternFill>
@@ -1483,34 +1477,6 @@
       <fill>
         <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1559,7 +1525,56 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -10431,15 +10446,15 @@
         <v>78</v>
       </c>
       <c r="D5" s="30">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -10619,36 +10634,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="60" t="s">
         <v>129</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="F2" s="54" t="s">
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="F2" s="60" t="s">
         <v>130</v>
       </c>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="J2" s="54" t="s">
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="J2" s="60" t="s">
         <v>131</v>
       </c>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="N2" s="54" t="s">
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="N2" s="60" t="s">
         <v>132</v>
       </c>
-      <c r="O2" s="54"/>
-      <c r="P2" s="54"/>
-      <c r="R2" s="54" t="s">
+      <c r="O2" s="60"/>
+      <c r="P2" s="60"/>
+      <c r="R2" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="S2" s="54"/>
-      <c r="T2" s="54"/>
-      <c r="V2" s="54" t="s">
+      <c r="S2" s="60"/>
+      <c r="T2" s="60"/>
+      <c r="V2" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="W2" s="54"/>
-      <c r="X2" s="54"/>
+      <c r="W2" s="60"/>
+      <c r="X2" s="60"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -12404,34 +12419,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="61" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="E2" s="51" t="s">
+      <c r="C2" s="61"/>
+      <c r="E2" s="57" t="s">
         <v>215</v>
       </c>
-      <c r="F2" s="51"/>
-      <c r="H2" s="51" t="s">
+      <c r="F2" s="57"/>
+      <c r="H2" s="57" t="s">
         <v>217</v>
       </c>
-      <c r="I2" s="51"/>
-      <c r="K2" s="51" t="s">
+      <c r="I2" s="57"/>
+      <c r="K2" s="57" t="s">
         <v>218</v>
       </c>
-      <c r="L2" s="51"/>
-      <c r="N2" s="51" t="s">
+      <c r="L2" s="57"/>
+      <c r="N2" s="57" t="s">
         <v>219</v>
       </c>
-      <c r="O2" s="51"/>
-      <c r="Q2" s="51" t="s">
+      <c r="O2" s="57"/>
+      <c r="Q2" s="57" t="s">
         <v>220</v>
       </c>
-      <c r="R2" s="51"/>
+      <c r="R2" s="57"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
       <c r="E3" s="32" t="s">
         <v>213</v>
       </c>
@@ -12820,34 +12835,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="62" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="E2" s="52" t="s">
+      <c r="C2" s="62"/>
+      <c r="E2" s="58" t="s">
         <v>221</v>
       </c>
-      <c r="F2" s="52"/>
-      <c r="H2" s="52" t="s">
+      <c r="F2" s="58"/>
+      <c r="H2" s="58" t="s">
         <v>222</v>
       </c>
-      <c r="I2" s="52"/>
-      <c r="K2" s="52" t="s">
+      <c r="I2" s="58"/>
+      <c r="K2" s="58" t="s">
         <v>223</v>
       </c>
-      <c r="L2" s="52"/>
-      <c r="N2" s="52" t="s">
+      <c r="L2" s="58"/>
+      <c r="N2" s="58" t="s">
         <v>224</v>
       </c>
-      <c r="O2" s="52"/>
-      <c r="Q2" s="52" t="s">
+      <c r="O2" s="58"/>
+      <c r="Q2" s="58" t="s">
         <v>225</v>
       </c>
-      <c r="R2" s="52"/>
+      <c r="R2" s="58"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
       <c r="E3" s="34" t="s">
         <v>213</v>
       </c>
@@ -13232,34 +13247,34 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A900FC-A692-B445-95C9-59E70352B291}">
-  <dimension ref="A2:AL52"/>
+  <dimension ref="A2:AN52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
     <col min="3" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="38" width="8.5" customWidth="1"/>
+    <col min="11" max="40" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
         <v>67</v>
       </c>
       <c r="E2"/>
       <c r="F2"/>
       <c r="G2"/>
-      <c r="L2" s="6" t="s">
+      <c r="N2" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="Q2" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="AB2" s="6"/>
-      <c r="AH2" s="6" t="s">
+      <c r="AD2" s="6"/>
+      <c r="AJ2" s="6" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
         <v>66</v>
       </c>
@@ -13268,21 +13283,21 @@
       </c>
       <c r="F3"/>
       <c r="G3"/>
-      <c r="O3" s="1" t="s">
+      <c r="Q3" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="P3" t="s">
+      <c r="R3" t="s">
         <v>58</v>
       </c>
-      <c r="AB3" s="14"/>
-      <c r="AH3" s="1" t="s">
+      <c r="AD3" s="14"/>
+      <c r="AJ3" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="AI3" t="s">
+      <c r="AK3" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
         <v>69</v>
       </c>
@@ -13291,240 +13306,248 @@
       </c>
       <c r="F4"/>
       <c r="G4"/>
-      <c r="L4" s="42"/>
-      <c r="M4" t="s">
+      <c r="N4" s="42"/>
+      <c r="O4" t="s">
         <v>161</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="Q4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="P4" t="s">
+      <c r="R4" t="s">
         <v>59</v>
       </c>
-      <c r="AB4" s="14"/>
-      <c r="AH4" s="1" t="s">
+      <c r="AD4" s="14"/>
+      <c r="AJ4" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="AI4" t="s">
+      <c r="AK4" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C5" s="1" t="s">
         <v>171</v>
       </c>
       <c r="D5" t="s">
         <v>191</v>
       </c>
-      <c r="L5" s="26"/>
-      <c r="M5" s="9" t="s">
+      <c r="N5" s="26"/>
+      <c r="O5" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="Q5" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="P5" s="9" t="s">
+      <c r="R5" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="AB5" s="14"/>
-      <c r="AH5" s="1" t="s">
+      <c r="AD5" s="14"/>
+      <c r="AJ5" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="AI5" s="9" t="s">
+      <c r="AK5" s="9" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C6" s="1" t="s">
         <v>201</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="L6" s="29"/>
-      <c r="M6" s="9" t="s">
+      <c r="N6" s="29"/>
+      <c r="O6" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="Q6" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="P6" t="s">
+      <c r="R6" t="s">
         <v>190</v>
       </c>
-      <c r="AC6" s="1"/>
-      <c r="AD6" s="1"/>
-    </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE6" s="1"/>
+      <c r="AF6" s="1"/>
+    </row>
+    <row r="7" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C7" s="1" t="s">
         <v>233</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="AC7" s="1"/>
-      <c r="AD7" s="1"/>
-    </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.2">
-      <c r="C9" s="45" t="s">
+      <c r="AE7" s="1"/>
+      <c r="AF7" s="1"/>
+    </row>
+    <row r="9" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="C9" s="51" t="s">
         <v>236</v>
       </c>
-      <c r="D9" s="45"/>
-      <c r="E9" s="45"/>
-      <c r="F9" s="45"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="45"/>
-      <c r="I9" s="45"/>
-      <c r="J9" s="45"/>
-      <c r="K9" s="45"/>
-      <c r="L9" s="45"/>
-      <c r="M9" s="45"/>
-      <c r="N9" s="45"/>
-      <c r="O9" s="45"/>
-      <c r="P9" s="45"/>
-      <c r="Q9" s="45"/>
-      <c r="R9" s="45"/>
-      <c r="S9" s="45"/>
-      <c r="T9" s="45"/>
-      <c r="U9" s="45"/>
-      <c r="V9" s="45"/>
-      <c r="W9" s="45"/>
-      <c r="X9" s="45"/>
-      <c r="Y9" s="45" t="s">
+      <c r="D9" s="51"/>
+      <c r="E9" s="51"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="51"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="51"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="51"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="51"/>
+      <c r="O9" s="51"/>
+      <c r="P9" s="51"/>
+      <c r="Q9" s="51"/>
+      <c r="R9" s="51"/>
+      <c r="S9" s="51"/>
+      <c r="T9" s="51"/>
+      <c r="U9" s="51"/>
+      <c r="V9" s="51"/>
+      <c r="W9" s="51"/>
+      <c r="X9" s="51"/>
+      <c r="Y9" s="51"/>
+      <c r="Z9" s="51"/>
+      <c r="AA9" s="51" t="s">
         <v>57</v>
       </c>
-      <c r="Z9" s="45"/>
-      <c r="AA9" s="45"/>
-      <c r="AB9" s="45"/>
-      <c r="AC9" s="45"/>
-      <c r="AD9" s="45"/>
-      <c r="AE9" s="45" t="s">
+      <c r="AB9" s="51"/>
+      <c r="AC9" s="51"/>
+      <c r="AD9" s="51"/>
+      <c r="AE9" s="51"/>
+      <c r="AF9" s="51"/>
+      <c r="AG9" s="51" t="s">
         <v>91</v>
       </c>
-      <c r="AF9" s="45"/>
-      <c r="AG9" s="45"/>
-      <c r="AH9" s="45"/>
-      <c r="AI9" s="45"/>
-      <c r="AJ9" s="45"/>
-      <c r="AK9" s="45"/>
-      <c r="AL9" s="45"/>
-    </row>
-    <row r="10" spans="1:38" ht="18" x14ac:dyDescent="0.25">
+      <c r="AH9" s="51"/>
+      <c r="AI9" s="51"/>
+      <c r="AJ9" s="51"/>
+      <c r="AK9" s="51"/>
+      <c r="AL9" s="51"/>
+      <c r="AM9" s="51"/>
+      <c r="AN9" s="51"/>
+    </row>
+    <row r="10" spans="1:40" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="C10" s="58" t="s">
+      <c r="C10" s="45" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="62" t="s">
+      <c r="D10" s="48" t="s">
         <v>189</v>
       </c>
-      <c r="E10" s="57" t="s">
+      <c r="E10" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="57" t="s">
+      <c r="F10" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="G10" s="58" t="s">
+      <c r="G10" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="H10" s="57" t="s">
+      <c r="H10" s="44" t="s">
         <v>72</v>
       </c>
-      <c r="I10" s="57" t="s">
+      <c r="I10" s="44" t="s">
         <v>71</v>
       </c>
-      <c r="J10" s="64" t="s">
+      <c r="J10" s="49" t="s">
         <v>79</v>
       </c>
-      <c r="K10" s="64" t="s">
+      <c r="K10" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="L10" s="63" t="s">
+      <c r="L10" s="49" t="s">
+        <v>238</v>
+      </c>
+      <c r="M10" s="49" t="s">
+        <v>239</v>
+      </c>
+      <c r="N10" s="21" t="s">
         <v>235</v>
       </c>
-      <c r="M10" s="21" t="s">
+      <c r="O10" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="N10" s="43" t="s">
+      <c r="P10" s="43" t="s">
         <v>211</v>
       </c>
-      <c r="O10" s="57" t="s">
+      <c r="Q10" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="P10" s="57" t="s">
+      <c r="R10" s="44" t="s">
         <v>172</v>
       </c>
-      <c r="Q10" s="57" t="s">
+      <c r="S10" s="44" t="s">
         <v>173</v>
       </c>
-      <c r="R10" s="57" t="s">
+      <c r="T10" s="44" t="s">
         <v>174</v>
       </c>
-      <c r="S10" s="57" t="s">
+      <c r="U10" s="44" t="s">
         <v>175</v>
       </c>
-      <c r="T10" s="57" t="s">
+      <c r="V10" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="U10" s="57" t="s">
+      <c r="W10" s="44" t="s">
         <v>206</v>
       </c>
-      <c r="V10" s="57" t="s">
+      <c r="X10" s="44" t="s">
         <v>208</v>
       </c>
-      <c r="W10" s="57" t="s">
+      <c r="Y10" s="44" t="s">
         <v>209</v>
       </c>
-      <c r="X10" s="57" t="s">
+      <c r="Z10" s="44" t="s">
         <v>210</v>
       </c>
-      <c r="Y10" s="59" t="s">
+      <c r="AA10" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="Z10" s="59" t="s">
+      <c r="AB10" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="AA10" s="60" t="s">
+      <c r="AC10" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="AB10" s="59" t="s">
+      <c r="AD10" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="AC10" s="59" t="s">
+      <c r="AE10" s="46" t="s">
         <v>80</v>
       </c>
-      <c r="AD10" s="60" t="s">
+      <c r="AF10" s="47" t="s">
         <v>136</v>
       </c>
-      <c r="AE10" s="23" t="s">
+      <c r="AG10" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AF10" s="23" t="s">
+      <c r="AH10" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AG10" s="23" t="s">
+      <c r="AI10" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="AH10" s="23" t="s">
+      <c r="AJ10" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="AI10" s="23" t="s">
+      <c r="AK10" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="AJ10" s="23" t="s">
+      <c r="AL10" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="AK10" s="23" t="s">
+      <c r="AM10" s="23" t="s">
         <v>205</v>
       </c>
-      <c r="AL10" s="23" t="s">
+      <c r="AN10" s="23" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>1</v>
       </c>
@@ -13565,8 +13588,10 @@
       <c r="AJ11" s="3"/>
       <c r="AK11" s="3"/>
       <c r="AL11" s="3"/>
-    </row>
-    <row r="12" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM11" s="3"/>
+      <c r="AN11" s="3"/>
+    </row>
+    <row r="12" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -13605,10 +13630,12 @@
       <c r="AH12" s="3"/>
       <c r="AI12" s="3"/>
       <c r="AJ12" s="3"/>
-      <c r="AK12" s="18"/>
-      <c r="AL12" s="19"/>
-    </row>
-    <row r="13" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AK12" s="3"/>
+      <c r="AL12" s="3"/>
+      <c r="AM12" s="18"/>
+      <c r="AN12" s="19"/>
+    </row>
+    <row r="13" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>3</v>
       </c>
@@ -13647,10 +13674,12 @@
       <c r="AH13" s="3"/>
       <c r="AI13" s="3"/>
       <c r="AJ13" s="3"/>
-      <c r="AK13" s="18"/>
-      <c r="AL13" s="19"/>
-    </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AK13" s="3"/>
+      <c r="AL13" s="3"/>
+      <c r="AM13" s="18"/>
+      <c r="AN13" s="19"/>
+    </row>
+    <row r="14" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>4</v>
       </c>
@@ -13691,8 +13720,10 @@
       <c r="AJ14" s="3"/>
       <c r="AK14" s="3"/>
       <c r="AL14" s="3"/>
-    </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM14" s="3"/>
+      <c r="AN14" s="3"/>
+    </row>
+    <row r="15" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>5</v>
       </c>
@@ -13733,8 +13764,10 @@
       <c r="AJ15" s="3"/>
       <c r="AK15" s="3"/>
       <c r="AL15" s="3"/>
-    </row>
-    <row r="16" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM15" s="3"/>
+      <c r="AN15" s="3"/>
+    </row>
+    <row r="16" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>6</v>
       </c>
@@ -13775,8 +13808,10 @@
       <c r="AJ16" s="3"/>
       <c r="AK16" s="3"/>
       <c r="AL16" s="3"/>
-    </row>
-    <row r="17" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM16" s="3"/>
+      <c r="AN16" s="3"/>
+    </row>
+    <row r="17" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>7</v>
       </c>
@@ -13817,8 +13852,10 @@
       <c r="AJ17" s="3"/>
       <c r="AK17" s="3"/>
       <c r="AL17" s="3"/>
-    </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM17" s="3"/>
+      <c r="AN17" s="3"/>
+    </row>
+    <row r="18" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>8</v>
       </c>
@@ -13859,8 +13896,10 @@
       <c r="AJ18" s="3"/>
       <c r="AK18" s="3"/>
       <c r="AL18" s="3"/>
-    </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM18" s="3"/>
+      <c r="AN18" s="3"/>
+    </row>
+    <row r="19" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>9</v>
       </c>
@@ -13901,8 +13940,10 @@
       <c r="AJ19" s="3"/>
       <c r="AK19" s="3"/>
       <c r="AL19" s="3"/>
-    </row>
-    <row r="20" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM19" s="3"/>
+      <c r="AN19" s="3"/>
+    </row>
+    <row r="20" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>10</v>
       </c>
@@ -13943,8 +13984,10 @@
       <c r="AJ20" s="3"/>
       <c r="AK20" s="3"/>
       <c r="AL20" s="3"/>
-    </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM20" s="3"/>
+      <c r="AN20" s="3"/>
+    </row>
+    <row r="21" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>11</v>
       </c>
@@ -13985,8 +14028,10 @@
       <c r="AJ21" s="3"/>
       <c r="AK21" s="3"/>
       <c r="AL21" s="3"/>
-    </row>
-    <row r="22" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM21" s="3"/>
+      <c r="AN21" s="3"/>
+    </row>
+    <row r="22" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>12</v>
       </c>
@@ -14027,8 +14072,10 @@
       <c r="AJ22" s="3"/>
       <c r="AK22" s="3"/>
       <c r="AL22" s="3"/>
-    </row>
-    <row r="23" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM22" s="3"/>
+      <c r="AN22" s="3"/>
+    </row>
+    <row r="23" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>13</v>
       </c>
@@ -14069,8 +14116,10 @@
       <c r="AJ23" s="3"/>
       <c r="AK23" s="3"/>
       <c r="AL23" s="3"/>
-    </row>
-    <row r="24" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM23" s="3"/>
+      <c r="AN23" s="3"/>
+    </row>
+    <row r="24" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>14</v>
       </c>
@@ -14111,8 +14160,10 @@
       <c r="AJ24" s="3"/>
       <c r="AK24" s="3"/>
       <c r="AL24" s="3"/>
-    </row>
-    <row r="25" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM24" s="3"/>
+      <c r="AN24" s="3"/>
+    </row>
+    <row r="25" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>15</v>
       </c>
@@ -14153,8 +14204,10 @@
       <c r="AJ25" s="3"/>
       <c r="AK25" s="3"/>
       <c r="AL25" s="3"/>
-    </row>
-    <row r="26" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM25" s="3"/>
+      <c r="AN25" s="3"/>
+    </row>
+    <row r="26" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -14183,8 +14236,10 @@
       <c r="AJ26" s="1"/>
       <c r="AK26" s="1"/>
       <c r="AL26" s="1"/>
-    </row>
-    <row r="27" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM26" s="1"/>
+      <c r="AN26" s="1"/>
+    </row>
+    <row r="27" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -14205,8 +14260,10 @@
       <c r="AB27" s="1"/>
       <c r="AC27" s="1"/>
       <c r="AD27" s="1"/>
-    </row>
-    <row r="28" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE27" s="1"/>
+      <c r="AF27" s="1"/>
+    </row>
+    <row r="28" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -14227,8 +14284,10 @@
       <c r="AB28" s="1"/>
       <c r="AC28" s="1"/>
       <c r="AD28" s="1"/>
-    </row>
-    <row r="29" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE28" s="1"/>
+      <c r="AF28" s="1"/>
+    </row>
+    <row r="29" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -14249,8 +14308,10 @@
       <c r="AB29" s="1"/>
       <c r="AC29" s="1"/>
       <c r="AD29" s="1"/>
-    </row>
-    <row r="30" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE29" s="1"/>
+      <c r="AF29" s="1"/>
+    </row>
+    <row r="30" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -14271,8 +14332,10 @@
       <c r="AB30" s="1"/>
       <c r="AC30" s="1"/>
       <c r="AD30" s="1"/>
-    </row>
-    <row r="31" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE30" s="1"/>
+      <c r="AF30" s="1"/>
+    </row>
+    <row r="31" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -14293,8 +14356,10 @@
       <c r="AB31" s="1"/>
       <c r="AC31" s="1"/>
       <c r="AD31" s="1"/>
-    </row>
-    <row r="32" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE31" s="1"/>
+      <c r="AF31" s="1"/>
+    </row>
+    <row r="32" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -14315,8 +14380,10 @@
       <c r="AB32" s="1"/>
       <c r="AC32" s="1"/>
       <c r="AD32" s="1"/>
-    </row>
-    <row r="33" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE32" s="1"/>
+      <c r="AF32" s="1"/>
+    </row>
+    <row r="33" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
@@ -14337,8 +14404,10 @@
       <c r="AB33" s="1"/>
       <c r="AC33" s="1"/>
       <c r="AD33" s="1"/>
-    </row>
-    <row r="34" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE33" s="1"/>
+      <c r="AF33" s="1"/>
+    </row>
+    <row r="34" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
@@ -14359,8 +14428,10 @@
       <c r="AB34" s="1"/>
       <c r="AC34" s="1"/>
       <c r="AD34" s="1"/>
-    </row>
-    <row r="35" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE34" s="1"/>
+      <c r="AF34" s="1"/>
+    </row>
+    <row r="35" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
@@ -14381,8 +14452,10 @@
       <c r="AB35" s="1"/>
       <c r="AC35" s="1"/>
       <c r="AD35" s="1"/>
-    </row>
-    <row r="36" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE35" s="1"/>
+      <c r="AF35" s="1"/>
+    </row>
+    <row r="36" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -14403,8 +14476,10 @@
       <c r="AB36" s="1"/>
       <c r="AC36" s="1"/>
       <c r="AD36" s="1"/>
-    </row>
-    <row r="37" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE36" s="1"/>
+      <c r="AF36" s="1"/>
+    </row>
+    <row r="37" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
@@ -14425,8 +14500,10 @@
       <c r="AB37" s="1"/>
       <c r="AC37" s="1"/>
       <c r="AD37" s="1"/>
-    </row>
-    <row r="38" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE37" s="1"/>
+      <c r="AF37" s="1"/>
+    </row>
+    <row r="38" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
@@ -14447,8 +14524,10 @@
       <c r="AB38" s="1"/>
       <c r="AC38" s="1"/>
       <c r="AD38" s="1"/>
-    </row>
-    <row r="39" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE38" s="1"/>
+      <c r="AF38" s="1"/>
+    </row>
+    <row r="39" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -14469,8 +14548,10 @@
       <c r="AB39" s="1"/>
       <c r="AC39" s="1"/>
       <c r="AD39" s="1"/>
-    </row>
-    <row r="40" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE39" s="1"/>
+      <c r="AF39" s="1"/>
+    </row>
+    <row r="40" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
@@ -14491,8 +14572,10 @@
       <c r="AB40" s="1"/>
       <c r="AC40" s="1"/>
       <c r="AD40" s="1"/>
-    </row>
-    <row r="41" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE40" s="1"/>
+      <c r="AF40" s="1"/>
+    </row>
+    <row r="41" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
@@ -14513,8 +14596,10 @@
       <c r="AB41" s="1"/>
       <c r="AC41" s="1"/>
       <c r="AD41" s="1"/>
-    </row>
-    <row r="42" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE41" s="1"/>
+      <c r="AF41" s="1"/>
+    </row>
+    <row r="42" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
@@ -14535,8 +14620,10 @@
       <c r="AB42" s="1"/>
       <c r="AC42" s="1"/>
       <c r="AD42" s="1"/>
-    </row>
-    <row r="43" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE42" s="1"/>
+      <c r="AF42" s="1"/>
+    </row>
+    <row r="43" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
@@ -14557,8 +14644,10 @@
       <c r="AB43" s="1"/>
       <c r="AC43" s="1"/>
       <c r="AD43" s="1"/>
-    </row>
-    <row r="44" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE43" s="1"/>
+      <c r="AF43" s="1"/>
+    </row>
+    <row r="44" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
@@ -14579,8 +14668,10 @@
       <c r="AB44" s="1"/>
       <c r="AC44" s="1"/>
       <c r="AD44" s="1"/>
-    </row>
-    <row r="45" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE44" s="1"/>
+      <c r="AF44" s="1"/>
+    </row>
+    <row r="45" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
@@ -14601,8 +14692,10 @@
       <c r="AB45" s="1"/>
       <c r="AC45" s="1"/>
       <c r="AD45" s="1"/>
-    </row>
-    <row r="46" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE45" s="1"/>
+      <c r="AF45" s="1"/>
+    </row>
+    <row r="46" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
@@ -14623,8 +14716,10 @@
       <c r="AB46" s="1"/>
       <c r="AC46" s="1"/>
       <c r="AD46" s="1"/>
-    </row>
-    <row r="47" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE46" s="1"/>
+      <c r="AF46" s="1"/>
+    </row>
+    <row r="47" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
       <c r="M47" s="1"/>
@@ -14645,8 +14740,10 @@
       <c r="AB47" s="1"/>
       <c r="AC47" s="1"/>
       <c r="AD47" s="1"/>
-    </row>
-    <row r="48" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE47" s="1"/>
+      <c r="AF47" s="1"/>
+    </row>
+    <row r="48" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
@@ -14667,8 +14764,10 @@
       <c r="AB48" s="1"/>
       <c r="AC48" s="1"/>
       <c r="AD48" s="1"/>
-    </row>
-    <row r="49" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE48" s="1"/>
+      <c r="AF48" s="1"/>
+    </row>
+    <row r="49" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
@@ -14689,8 +14788,10 @@
       <c r="AB49" s="1"/>
       <c r="AC49" s="1"/>
       <c r="AD49" s="1"/>
-    </row>
-    <row r="50" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE49" s="1"/>
+      <c r="AF49" s="1"/>
+    </row>
+    <row r="50" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K50" s="1"/>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
@@ -14711,8 +14812,10 @@
       <c r="AB50" s="1"/>
       <c r="AC50" s="1"/>
       <c r="AD50" s="1"/>
-    </row>
-    <row r="51" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE50" s="1"/>
+      <c r="AF50" s="1"/>
+    </row>
+    <row r="51" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
@@ -14733,8 +14836,10 @@
       <c r="AB51" s="1"/>
       <c r="AC51" s="1"/>
       <c r="AD51" s="1"/>
-    </row>
-    <row r="52" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE51" s="1"/>
+      <c r="AF51" s="1"/>
+    </row>
+    <row r="52" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
@@ -14755,100 +14860,107 @@
       <c r="AB52" s="1"/>
       <c r="AC52" s="1"/>
       <c r="AD52" s="1"/>
+      <c r="AE52" s="1"/>
+      <c r="AF52" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="Y9:AD9"/>
-    <mergeCell ref="AE9:AL9"/>
-    <mergeCell ref="C9:X9"/>
+    <mergeCell ref="AA9:AF9"/>
+    <mergeCell ref="AG9:AN9"/>
+    <mergeCell ref="C9:Z9"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:K52 Z11:AD52">
-    <cfRule type="expression" dxfId="5" priority="1">
+  <conditionalFormatting sqref="L11:M52">
+    <cfRule type="expression" dxfId="5" priority="17">
+      <formula>AND($Q11&lt;&gt;"",$Q11&lt;&gt;"piezo",$Q11&lt;&gt;"seep")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F11:K52 AB11:AF52">
+    <cfRule type="expression" dxfId="18" priority="1">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="17" priority="2">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F11:N52">
+    <cfRule type="expression" dxfId="16" priority="14">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="15" priority="3">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="5" priority="4">
+    <cfRule type="expression" dxfId="14" priority="4">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="5" priority="5">
+  <conditionalFormatting sqref="J11:M52">
+    <cfRule type="expression" dxfId="13" priority="5">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:T52">
-    <cfRule type="expression" dxfId="5" priority="6">
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="12" priority="15">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R11:R52">
+    <cfRule type="expression" dxfId="11" priority="8">
+      <formula>AND($Q11&lt;&gt;"",$Q11&lt;&gt;"ru")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S11:V52">
+    <cfRule type="expression" dxfId="10" priority="6">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U11:X52">
-    <cfRule type="expression" dxfId="5" priority="7">
+  <conditionalFormatting sqref="W11:Z52">
+    <cfRule type="expression" dxfId="9" priority="7">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P11:P52">
-    <cfRule type="expression" dxfId="5" priority="8">
-      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
+  <conditionalFormatting sqref="AB11:AF52">
+    <cfRule type="expression" dxfId="8" priority="16">
+      <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA11:AA52">
-    <cfRule type="expression" dxfId="5" priority="9">
+  <conditionalFormatting sqref="AC11:AC52">
+    <cfRule type="expression" dxfId="7" priority="9">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB11:AB52">
-    <cfRule type="expression" dxfId="5" priority="10">
+  <conditionalFormatting sqref="AD11:AD52">
+    <cfRule type="expression" dxfId="6" priority="10">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC11:AD52">
+  <conditionalFormatting sqref="AE11:AF52">
     <cfRule type="expression" dxfId="5" priority="11">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI11:AJ52">
-    <cfRule type="expression" dxfId="5" priority="12">
-      <formula>OR($AH11="vg",$AH11="gard")</formula>
+  <conditionalFormatting sqref="AK11:AL52">
+    <cfRule type="expression" dxfId="4" priority="12">
+      <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="5" priority="13">
-      <formula>$AH11="lf"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F11:L52">
-    <cfRule type="expression" dxfId="5" priority="14">
-      <formula>$E11="elastic"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O11:P52">
-    <cfRule type="expression" dxfId="5" priority="15">
-      <formula>$E11="elastic"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z11:AD52">
-    <cfRule type="expression" dxfId="5" priority="16">
-      <formula>$E11="elastic"</formula>
+  <conditionalFormatting sqref="AM11:AN52">
+    <cfRule type="expression" dxfId="3" priority="13">
+      <formula>$AJ11="lf"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11:E52" xr:uid="{374AFD2C-B540-DD4B-A245-8B781F76E64C}">
       <formula1>$C$3:$C$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH11:AH102" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
-      <formula1>$AH$3:$AH$5</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ11:AJ102" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
+      <formula1>$AJ$3:$AJ$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O11:O52" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
-      <formula1>$O$3:$O$6</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q11:Q52" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
+      <formula1>$Q$3:$Q$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14893,74 +15005,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="D4" s="48" t="s">
+      <c r="B4" s="52"/>
+      <c r="D4" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="G4" s="48" t="s">
+      <c r="E4" s="52"/>
+      <c r="G4" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="48"/>
-      <c r="J4" s="48" t="s">
+      <c r="H4" s="52"/>
+      <c r="J4" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="48"/>
-      <c r="M4" s="48" t="s">
+      <c r="K4" s="52"/>
+      <c r="M4" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="48"/>
-      <c r="P4" s="48" t="s">
+      <c r="N4" s="52"/>
+      <c r="P4" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="48"/>
+      <c r="Q4" s="52"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="48" t="s">
+      <c r="S4" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="48"/>
+      <c r="T4" s="52"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="48" t="s">
+      <c r="V4" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="48"/>
+      <c r="W4" s="52"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="48" t="s">
+      <c r="Y4" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="48"/>
+      <c r="Z4" s="52"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="48" t="s">
+      <c r="AB4" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="48"/>
-      <c r="AE4" s="48" t="s">
+      <c r="AC4" s="52"/>
+      <c r="AE4" s="52" t="s">
         <v>108</v>
       </c>
-      <c r="AF4" s="48"/>
+      <c r="AF4" s="52"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="48" t="s">
+      <c r="AH4" s="52" t="s">
         <v>109</v>
       </c>
-      <c r="AI4" s="48"/>
+      <c r="AI4" s="52"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="48" t="s">
+      <c r="AK4" s="52" t="s">
         <v>110</v>
       </c>
-      <c r="AL4" s="48"/>
+      <c r="AL4" s="52"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="48" t="s">
+      <c r="AN4" s="52" t="s">
         <v>111</v>
       </c>
-      <c r="AO4" s="48"/>
+      <c r="AO4" s="52"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="48" t="s">
+      <c r="AQ4" s="52" t="s">
         <v>112</v>
       </c>
-      <c r="AR4" s="48"/>
+      <c r="AR4" s="52"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
@@ -15063,89 +15175,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="46" t="str">
+      <c r="A6" s="53" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="47"/>
-      <c r="D6" s="46" t="str">
+      <c r="B6" s="54"/>
+      <c r="D6" s="53" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="47"/>
-      <c r="G6" s="46" t="str">
+      <c r="E6" s="54"/>
+      <c r="G6" s="53" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="47"/>
-      <c r="J6" s="46" t="str">
+      <c r="H6" s="54"/>
+      <c r="J6" s="53" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="47"/>
-      <c r="M6" s="46" t="str">
+      <c r="K6" s="54"/>
+      <c r="M6" s="53" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="47"/>
-      <c r="P6" s="46" t="str">
+      <c r="N6" s="54"/>
+      <c r="P6" s="53" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="47"/>
+      <c r="Q6" s="54"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="46" t="str">
+      <c r="S6" s="53" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="47"/>
+      <c r="T6" s="54"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="46" t="str">
+      <c r="V6" s="53" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="47"/>
+      <c r="W6" s="54"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="46" t="str">
+      <c r="Y6" s="53" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="47"/>
+      <c r="Z6" s="54"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="46" t="str">
+      <c r="AB6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="47"/>
-      <c r="AE6" s="46" t="str">
+      <c r="AC6" s="54"/>
+      <c r="AE6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="47"/>
+      <c r="AF6" s="54"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="46" t="str">
+      <c r="AH6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="47"/>
+      <c r="AI6" s="54"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="46" t="str">
+      <c r="AK6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="47"/>
+      <c r="AL6" s="54"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="46" t="str">
+      <c r="AN6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="47"/>
+      <c r="AO6" s="54"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="46" t="str">
+      <c r="AQ6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="47"/>
+      <c r="AR6" s="54"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -16049,36 +16161,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16116,74 +16228,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="52" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="D4" s="48" t="s">
+      <c r="B4" s="52"/>
+      <c r="D4" s="52" t="s">
         <v>138</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="G4" s="48" t="s">
+      <c r="E4" s="52"/>
+      <c r="G4" s="52" t="s">
         <v>139</v>
       </c>
-      <c r="H4" s="48"/>
-      <c r="J4" s="48" t="s">
+      <c r="H4" s="52"/>
+      <c r="J4" s="52" t="s">
         <v>140</v>
       </c>
-      <c r="K4" s="48"/>
-      <c r="M4" s="48" t="s">
+      <c r="K4" s="52"/>
+      <c r="M4" s="52" t="s">
         <v>141</v>
       </c>
-      <c r="N4" s="48"/>
-      <c r="P4" s="48" t="s">
+      <c r="N4" s="52"/>
+      <c r="P4" s="52" t="s">
         <v>142</v>
       </c>
-      <c r="Q4" s="48"/>
+      <c r="Q4" s="52"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="48" t="s">
+      <c r="S4" s="52" t="s">
         <v>143</v>
       </c>
-      <c r="T4" s="48"/>
+      <c r="T4" s="52"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="48" t="s">
+      <c r="V4" s="52" t="s">
         <v>144</v>
       </c>
-      <c r="W4" s="48"/>
+      <c r="W4" s="52"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="48" t="s">
+      <c r="Y4" s="52" t="s">
         <v>145</v>
       </c>
-      <c r="Z4" s="48"/>
+      <c r="Z4" s="52"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="48" t="s">
+      <c r="AB4" s="52" t="s">
         <v>146</v>
       </c>
-      <c r="AC4" s="48"/>
-      <c r="AE4" s="48" t="s">
+      <c r="AC4" s="52"/>
+      <c r="AE4" s="52" t="s">
         <v>147</v>
       </c>
-      <c r="AF4" s="48"/>
+      <c r="AF4" s="52"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="48" t="s">
+      <c r="AH4" s="52" t="s">
         <v>148</v>
       </c>
-      <c r="AI4" s="48"/>
+      <c r="AI4" s="52"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="48" t="s">
+      <c r="AK4" s="52" t="s">
         <v>149</v>
       </c>
-      <c r="AL4" s="48"/>
+      <c r="AL4" s="52"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="48" t="s">
+      <c r="AN4" s="52" t="s">
         <v>150</v>
       </c>
-      <c r="AO4" s="48"/>
+      <c r="AO4" s="52"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="48" t="s">
+      <c r="AQ4" s="52" t="s">
         <v>151</v>
       </c>
-      <c r="AR4" s="48"/>
+      <c r="AR4" s="52"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
@@ -16286,89 +16398,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="49" t="str">
+      <c r="A6" s="55" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="50"/>
-      <c r="D6" s="49" t="str">
+      <c r="B6" s="56"/>
+      <c r="D6" s="55" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="50"/>
-      <c r="G6" s="49" t="str">
+      <c r="E6" s="56"/>
+      <c r="G6" s="55" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="50"/>
-      <c r="J6" s="49" t="str">
+      <c r="H6" s="56"/>
+      <c r="J6" s="55" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="50"/>
-      <c r="M6" s="49" t="str">
+      <c r="K6" s="56"/>
+      <c r="M6" s="55" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="50"/>
-      <c r="P6" s="49" t="str">
+      <c r="N6" s="56"/>
+      <c r="P6" s="55" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="50"/>
+      <c r="Q6" s="56"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="49" t="str">
+      <c r="S6" s="55" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="50"/>
+      <c r="T6" s="56"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="49" t="str">
+      <c r="V6" s="55" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="50"/>
+      <c r="W6" s="56"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="49" t="str">
+      <c r="Y6" s="55" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="50"/>
+      <c r="Z6" s="56"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="49" t="str">
+      <c r="AB6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="50"/>
-      <c r="AE6" s="49" t="str">
+      <c r="AC6" s="56"/>
+      <c r="AE6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="50"/>
+      <c r="AF6" s="56"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="49" t="str">
+      <c r="AH6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="50"/>
+      <c r="AI6" s="56"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="49" t="str">
+      <c r="AK6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="50"/>
+      <c r="AL6" s="56"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="49" t="str">
+      <c r="AN6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="50"/>
+      <c r="AO6" s="56"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="49" t="str">
+      <c r="AQ6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="50"/>
+      <c r="AR6" s="56"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -17272,12 +17384,14 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -17294,14 +17408,12 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17317,14 +17429,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="57" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="D2" s="52" t="s">
+      <c r="B2" s="57"/>
+      <c r="D2" s="58" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="52"/>
+      <c r="E2" s="58"/>
       <c r="G2" s="22" t="s">
         <v>82</v>
       </c>
@@ -17895,36 +18007,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="F2" s="53" t="s">
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="F2" s="59" t="s">
         <v>122</v>
       </c>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="J2" s="53" t="s">
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="J2" s="59" t="s">
         <v>123</v>
       </c>
-      <c r="K2" s="53"/>
-      <c r="L2" s="53"/>
-      <c r="N2" s="53" t="s">
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="N2" s="59" t="s">
         <v>124</v>
       </c>
-      <c r="O2" s="53"/>
-      <c r="P2" s="53"/>
-      <c r="R2" s="53" t="s">
+      <c r="O2" s="59"/>
+      <c r="P2" s="59"/>
+      <c r="R2" s="59" t="s">
         <v>125</v>
       </c>
-      <c r="S2" s="53"/>
-      <c r="T2" s="53"/>
-      <c r="V2" s="53" t="s">
+      <c r="S2" s="59"/>
+      <c r="T2" s="59"/>
+      <c r="V2" s="59" t="s">
         <v>126</v>
       </c>
-      <c r="W2" s="53"/>
-      <c r="X2" s="53"/>
+      <c r="W2" s="59"/>
+      <c r="X2" s="59"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">

</xml_diff>

<commit_message>
resources: sync bundled input_template.xlsx to v17 master (phi_b/s_cap at Q:R)
Byte-copy of docs/inputs/input_template.xlsx (the editable master, committed in
710e968) over the package-shipped copy so the two stay byte-identical, as the
run_tests.py check requires. The bundled copy is the save skeleton for library-
only / no-docs installs (default_template_path); it was stale (pre-relocation).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/xslope/resources/input_template.xlsx
+++ b/xslope/resources/input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9AE3CBE-0B2A-ED44-BB50-AACC6A5490D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920EFD39-E0D9-5841-8A8C-9199354BBCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="35040" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
@@ -1421,13 +1421,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1458,7 +1458,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="22">
     <dxf>
       <fill>
         <patternFill>
@@ -1477,6 +1477,27 @@
       <fill>
         <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -13263,10 +13284,10 @@
       <c r="E2"/>
       <c r="F2"/>
       <c r="G2"/>
-      <c r="N2" s="6" t="s">
+      <c r="L2" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="Q2" s="6" t="s">
+      <c r="O2" s="6" t="s">
         <v>170</v>
       </c>
       <c r="AD2" s="6"/>
@@ -13283,10 +13304,10 @@
       </c>
       <c r="F3"/>
       <c r="G3"/>
-      <c r="Q3" s="1" t="s">
+      <c r="O3" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="R3" t="s">
+      <c r="P3" t="s">
         <v>58</v>
       </c>
       <c r="AD3" s="14"/>
@@ -13306,14 +13327,14 @@
       </c>
       <c r="F4"/>
       <c r="G4"/>
-      <c r="N4" s="42"/>
-      <c r="O4" t="s">
+      <c r="L4" s="42"/>
+      <c r="M4" t="s">
         <v>161</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="O4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="R4" t="s">
+      <c r="P4" t="s">
         <v>59</v>
       </c>
       <c r="AD4" s="14"/>
@@ -13331,14 +13352,14 @@
       <c r="D5" t="s">
         <v>191</v>
       </c>
-      <c r="N5" s="26"/>
-      <c r="O5" s="9" t="s">
+      <c r="L5" s="26"/>
+      <c r="M5" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="Q5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="R5" s="9" t="s">
+      <c r="P5" s="9" t="s">
         <v>85</v>
       </c>
       <c r="AD5" s="14"/>
@@ -13356,14 +13377,14 @@
       <c r="D6" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="N6" s="29"/>
-      <c r="O6" s="9" t="s">
+      <c r="L6" s="29"/>
+      <c r="M6" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="Q6" s="1" t="s">
+      <c r="O6" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="R6" t="s">
+      <c r="P6" t="s">
         <v>190</v>
       </c>
       <c r="AE6" s="1"/>
@@ -13459,26 +13480,26 @@
       <c r="K10" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="L10" s="49" t="s">
+      <c r="L10" s="21" t="s">
+        <v>235</v>
+      </c>
+      <c r="M10" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="N10" s="43" t="s">
+        <v>211</v>
+      </c>
+      <c r="O10" s="44" t="s">
+        <v>84</v>
+      </c>
+      <c r="P10" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q10" s="44" t="s">
         <v>238</v>
       </c>
-      <c r="M10" s="49" t="s">
+      <c r="R10" s="44" t="s">
         <v>239</v>
-      </c>
-      <c r="N10" s="21" t="s">
-        <v>235</v>
-      </c>
-      <c r="O10" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="P10" s="43" t="s">
-        <v>211</v>
-      </c>
-      <c r="Q10" s="44" t="s">
-        <v>84</v>
-      </c>
-      <c r="R10" s="44" t="s">
-        <v>172</v>
       </c>
       <c r="S10" s="44" t="s">
         <v>173</v>
@@ -14869,87 +14890,97 @@
     <mergeCell ref="AG9:AN9"/>
     <mergeCell ref="C9:Z9"/>
   </mergeCells>
-  <conditionalFormatting sqref="L11:M52">
-    <cfRule type="expression" dxfId="5" priority="17">
-      <formula>AND($Q11&lt;&gt;"",$Q11&lt;&gt;"piezo",$Q11&lt;&gt;"seep")</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="F11:K52 AB11:AF52">
-    <cfRule type="expression" dxfId="18" priority="1">
+    <cfRule type="expression" dxfId="21" priority="4">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="2">
+    <cfRule type="expression" dxfId="20" priority="5">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F11:N52">
-    <cfRule type="expression" dxfId="16" priority="14">
+  <conditionalFormatting sqref="F11:L52">
+    <cfRule type="expression" dxfId="19" priority="17">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="18" priority="6">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="17" priority="7">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J11:M52">
-    <cfRule type="expression" dxfId="13" priority="5">
+  <conditionalFormatting sqref="J11:K52">
+    <cfRule type="expression" dxfId="16" priority="8">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O11:P52">
+    <cfRule type="expression" dxfId="15" priority="18">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P11:P52">
+    <cfRule type="expression" dxfId="14" priority="11">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S11:V52">
+    <cfRule type="expression" dxfId="13" priority="9">
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W11:Z52">
+    <cfRule type="expression" dxfId="12" priority="10">
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB11:AF52">
+    <cfRule type="expression" dxfId="11" priority="19">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC11:AC52">
+    <cfRule type="expression" dxfId="10" priority="12">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD11:AD52">
+    <cfRule type="expression" dxfId="9" priority="13">
+      <formula>$E11="mc"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE11:AF52">
+    <cfRule type="expression" dxfId="8" priority="14">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK11:AL52">
+    <cfRule type="expression" dxfId="7" priority="15">
+      <formula>OR($AJ11="vg",$AJ11="gard")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM11:AN52">
+    <cfRule type="expression" dxfId="6" priority="16">
+      <formula>$AJ11="lf"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="5" priority="2">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="12" priority="15">
-      <formula>$E11="elastic"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R11:R52">
-    <cfRule type="expression" dxfId="11" priority="8">
-      <formula>AND($Q11&lt;&gt;"",$Q11&lt;&gt;"ru")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S11:V52">
-    <cfRule type="expression" dxfId="10" priority="6">
-      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W11:Z52">
-    <cfRule type="expression" dxfId="9" priority="7">
-      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AB11:AF52">
-    <cfRule type="expression" dxfId="8" priority="16">
-      <formula>$E11="elastic"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC11:AC52">
-    <cfRule type="expression" dxfId="7" priority="9">
-      <formula>$E11="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="6" priority="10">
-      <formula>$E11="mc"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AE11:AF52">
-    <cfRule type="expression" dxfId="5" priority="11">
-      <formula>$E11="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="4" priority="12">
-      <formula>OR($AJ11="vg",$AJ11="gard")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM11:AN52">
-    <cfRule type="expression" dxfId="3" priority="13">
-      <formula>$AJ11="lf"</formula>
+    <cfRule type="expression" dxfId="3" priority="3">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -14959,8 +14990,8 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ11:AJ102" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
       <formula1>$AJ$3:$AJ$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q11:Q52" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
-      <formula1>$Q$3:$Q$6</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O11:O52" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
+      <formula1>$O$3:$O$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15005,74 +15036,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="D4" s="52" t="s">
+      <c r="B4" s="54"/>
+      <c r="D4" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="G4" s="52" t="s">
+      <c r="E4" s="54"/>
+      <c r="G4" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="52"/>
-      <c r="J4" s="52" t="s">
+      <c r="H4" s="54"/>
+      <c r="J4" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="52"/>
-      <c r="M4" s="52" t="s">
+      <c r="K4" s="54"/>
+      <c r="M4" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="52"/>
-      <c r="P4" s="52" t="s">
+      <c r="N4" s="54"/>
+      <c r="P4" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="52"/>
+      <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="52" t="s">
+      <c r="S4" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="52"/>
+      <c r="T4" s="54"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="52" t="s">
+      <c r="V4" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="52"/>
+      <c r="W4" s="54"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="52" t="s">
+      <c r="Y4" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="52"/>
+      <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="52" t="s">
+      <c r="AB4" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="52"/>
-      <c r="AE4" s="52" t="s">
+      <c r="AC4" s="54"/>
+      <c r="AE4" s="54" t="s">
         <v>108</v>
       </c>
-      <c r="AF4" s="52"/>
+      <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="52" t="s">
+      <c r="AH4" s="54" t="s">
         <v>109</v>
       </c>
-      <c r="AI4" s="52"/>
+      <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="52" t="s">
+      <c r="AK4" s="54" t="s">
         <v>110</v>
       </c>
-      <c r="AL4" s="52"/>
+      <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="52" t="s">
+      <c r="AN4" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="AO4" s="52"/>
+      <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="52" t="s">
+      <c r="AQ4" s="54" t="s">
         <v>112</v>
       </c>
-      <c r="AR4" s="52"/>
+      <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
@@ -15175,89 +15206,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="53" t="str">
+      <c r="A6" s="52" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="54"/>
-      <c r="D6" s="53" t="str">
+      <c r="B6" s="53"/>
+      <c r="D6" s="52" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="54"/>
-      <c r="G6" s="53" t="str">
+      <c r="E6" s="53"/>
+      <c r="G6" s="52" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="54"/>
-      <c r="J6" s="53" t="str">
+      <c r="H6" s="53"/>
+      <c r="J6" s="52" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="54"/>
-      <c r="M6" s="53" t="str">
+      <c r="K6" s="53"/>
+      <c r="M6" s="52" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="54"/>
-      <c r="P6" s="53" t="str">
+      <c r="N6" s="53"/>
+      <c r="P6" s="52" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="54"/>
+      <c r="Q6" s="53"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="53" t="str">
+      <c r="S6" s="52" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="54"/>
+      <c r="T6" s="53"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="53" t="str">
+      <c r="V6" s="52" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="54"/>
+      <c r="W6" s="53"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="53" t="str">
+      <c r="Y6" s="52" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="54"/>
+      <c r="Z6" s="53"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="53" t="str">
+      <c r="AB6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="54"/>
-      <c r="AE6" s="53" t="str">
+      <c r="AC6" s="53"/>
+      <c r="AE6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="54"/>
+      <c r="AF6" s="53"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="53" t="str">
+      <c r="AH6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="54"/>
+      <c r="AI6" s="53"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="53" t="str">
+      <c r="AK6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="54"/>
+      <c r="AL6" s="53"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="53" t="str">
+      <c r="AN6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="54"/>
+      <c r="AO6" s="53"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="53" t="str">
+      <c r="AQ6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="54"/>
+      <c r="AR6" s="53"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -16161,36 +16192,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16228,74 +16259,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="54" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="D4" s="52" t="s">
+      <c r="B4" s="54"/>
+      <c r="D4" s="54" t="s">
         <v>138</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="G4" s="52" t="s">
+      <c r="E4" s="54"/>
+      <c r="G4" s="54" t="s">
         <v>139</v>
       </c>
-      <c r="H4" s="52"/>
-      <c r="J4" s="52" t="s">
+      <c r="H4" s="54"/>
+      <c r="J4" s="54" t="s">
         <v>140</v>
       </c>
-      <c r="K4" s="52"/>
-      <c r="M4" s="52" t="s">
+      <c r="K4" s="54"/>
+      <c r="M4" s="54" t="s">
         <v>141</v>
       </c>
-      <c r="N4" s="52"/>
-      <c r="P4" s="52" t="s">
+      <c r="N4" s="54"/>
+      <c r="P4" s="54" t="s">
         <v>142</v>
       </c>
-      <c r="Q4" s="52"/>
+      <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="52" t="s">
+      <c r="S4" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="T4" s="52"/>
+      <c r="T4" s="54"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="52" t="s">
+      <c r="V4" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="W4" s="52"/>
+      <c r="W4" s="54"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="52" t="s">
+      <c r="Y4" s="54" t="s">
         <v>145</v>
       </c>
-      <c r="Z4" s="52"/>
+      <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="52" t="s">
+      <c r="AB4" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="AC4" s="52"/>
-      <c r="AE4" s="52" t="s">
+      <c r="AC4" s="54"/>
+      <c r="AE4" s="54" t="s">
         <v>147</v>
       </c>
-      <c r="AF4" s="52"/>
+      <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="52" t="s">
+      <c r="AH4" s="54" t="s">
         <v>148</v>
       </c>
-      <c r="AI4" s="52"/>
+      <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="52" t="s">
+      <c r="AK4" s="54" t="s">
         <v>149</v>
       </c>
-      <c r="AL4" s="52"/>
+      <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="52" t="s">
+      <c r="AN4" s="54" t="s">
         <v>150</v>
       </c>
-      <c r="AO4" s="52"/>
+      <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="52" t="s">
+      <c r="AQ4" s="54" t="s">
         <v>151</v>
       </c>
-      <c r="AR4" s="52"/>
+      <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
@@ -17384,14 +17415,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -17408,12 +17437,14 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(resources): sync bundled input_template.xlsx to v18 master
Byte-copy docs/inputs/input_template.xlsx (v18: units/time selectors,
tseep sheet, mat Ss/Sy, series BCs) into the wheel-bundled copy so the
template_sync guard is green again. The bundled resource lagged at v17
after the v18 master promotion (flagged by the docs lane); this closes
that ripple gap. filecmp byte-identical; no content change vs master.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/xslope/resources/input_template.xlsx
+++ b/xslope/resources/input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920EFD39-E0D9-5841-8A8C-9199354BBCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D06D1B-9F8B-4A48-B6E0-097F17D68253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="35040" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="34200" windowHeight="19900" activeTab="15" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -28,12 +28,13 @@
     <sheet name="lloads" sheetId="17" r:id="rId13"/>
     <sheet name="seep bc" sheetId="11" r:id="rId14"/>
     <sheet name="seep bc (2)" sheetId="14" r:id="rId15"/>
+    <sheet name="tseep" sheetId="19" r:id="rId16"/>
   </sheets>
   <definedNames>
-    <definedName name="crack_depth">main!$D$9</definedName>
-    <definedName name="crack_depth_water">main!$D$10</definedName>
-    <definedName name="gamma_w">main!$D$8</definedName>
-    <definedName name="k">main!$D$11</definedName>
+    <definedName name="crack_depth">main!$D$11</definedName>
+    <definedName name="crack_depth_water">main!$D$12</definedName>
+    <definedName name="gamma_w">main!$D$10</definedName>
+    <definedName name="k">main!$D$13</definedName>
     <definedName name="max_depth" localSheetId="4">polygon!#REF!</definedName>
     <definedName name="max_depth">profile!$B$2</definedName>
     <definedName name="mesh">mat!#REF!</definedName>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="265">
   <si>
     <t>X</t>
   </si>
@@ -947,6 +948,81 @@
   </si>
   <si>
     <t>s_cap</t>
+  </si>
+  <si>
+    <t>Unit Options:</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>Imperial</t>
+  </si>
+  <si>
+    <t>Units:</t>
+  </si>
+  <si>
+    <t>Time Units:</t>
+  </si>
+  <si>
+    <t>sec</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>hr</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>Time:</t>
+  </si>
+  <si>
+    <t>t1</t>
+  </si>
+  <si>
+    <t>t2</t>
+  </si>
+  <si>
+    <t>t3</t>
+  </si>
+  <si>
+    <t>t4</t>
+  </si>
+  <si>
+    <t>t5</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>save_interval:</t>
+  </si>
+  <si>
+    <t>duration:</t>
+  </si>
+  <si>
+    <t>stage_1:</t>
+  </si>
+  <si>
+    <t>stage_2:</t>
+  </si>
+  <si>
+    <t>tseep</t>
+  </si>
+  <si>
+    <t>Transient seepage boundary conditions and run options</t>
+  </si>
+  <si>
+    <t>Ss</t>
+  </si>
+  <si>
+    <t>Sy</t>
+  </si>
+  <si>
+    <t>save_times</t>
   </si>
 </sst>
 </file>
@@ -1096,7 +1172,7 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1193,6 +1269,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="7">
     <border>
@@ -1280,7 +1362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1415,6 +1497,9 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1458,7 +1543,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill>
@@ -1477,13 +1562,6 @@
       <fill>
         <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -8961,6 +9039,499 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>tseep!$C$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>t1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>tseep!$B$3:$B$100</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="98"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>tseep!$C$3:$C$100</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="98"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-538B-9247-859A-D6EC9732CE9B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>tseep!$D$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>t2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>tseep!$B$3:$B$100</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="98"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>tseep!$D$3:$D$100</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="98"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-538B-9247-859A-D6EC9732CE9B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>tseep!$E$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>t3</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>tseep!$B$3:$B$100</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="98"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>tseep!$E$3:$E$100</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="98"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-538B-9247-859A-D6EC9732CE9B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>tseep!$F$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>t4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>tseep!$B$3:$B$100</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="98"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>tseep!$F$3:$F$100</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="98"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-538B-9247-859A-D6EC9732CE9B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>tseep!$G$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>t5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>tseep!$B$3:$B$100</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="98"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>tseep!$G$3:$G$100</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="98"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-538B-9247-859A-D6EC9732CE9B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="782614975"/>
+        <c:axId val="782616767"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="782614975"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="782616767"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="782616767"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="782614975"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -9001,7 +9572,563 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -10125,6 +11252,47 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>99785</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>88901</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>299357</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>99787</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7655F65D-6FA7-DB16-246F-5BDA3120EC02}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -10442,7 +11610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71FAED0A-C8CC-8343-BA2E-B8E4255891E7}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.6640625" customWidth="1"/>
@@ -10467,15 +11635,15 @@
         <v>78</v>
       </c>
       <c r="D5" s="30">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="50"/>
-      <c r="D7" s="50"/>
+      <c r="C7" s="51"/>
+      <c r="D7" s="51"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -10485,10 +11653,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C8" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" s="1">
-        <v>62.4</v>
+        <v>243</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>242</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>113</v>
@@ -10499,10 +11667,10 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C9" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0</v>
+        <v>249</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>248</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>19</v>
@@ -10513,10 +11681,10 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C10" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D10" s="1">
-        <v>0</v>
+        <v>62.4</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>17</v>
@@ -10528,7 +11696,7 @@
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B11" s="1"/>
       <c r="C11" s="14" t="s">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="D11" s="1">
         <v>0</v>
@@ -10541,6 +11709,12 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C12" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
       <c r="F12" s="1" t="s">
         <v>21</v>
       </c>
@@ -10549,6 +11723,12 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C13" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0</v>
+      </c>
       <c r="F13" s="1" t="s">
         <v>23</v>
       </c>
@@ -10621,16 +11801,72 @@
         <v>118</v>
       </c>
     </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="F22" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="G22" t="s">
+        <v>261</v>
+      </c>
+    </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="1"/>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="1"/>
+    </row>
+    <row r="49" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D49" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="50" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D50" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="51" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D51" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="53" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D53" s="1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="54" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D54" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="55" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D55" s="1" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="56" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D56" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="57" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D57" s="1" t="s">
+        <v>248</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B7:D7"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{BAE3FC11-E776-8E44-B1AE-D9B052583E4F}">
+      <formula1>$D$50:$D$51</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9" xr:uid="{73E87265-AF9F-0944-800E-CFF30E3B4CA4}">
+      <formula1>$D$54:$D$57</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -10655,36 +11891,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="60" t="s">
+      <c r="B2" s="61" t="s">
         <v>129</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="F2" s="60" t="s">
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="F2" s="61" t="s">
         <v>130</v>
       </c>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="J2" s="60" t="s">
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="J2" s="61" t="s">
         <v>131</v>
       </c>
-      <c r="K2" s="60"/>
-      <c r="L2" s="60"/>
-      <c r="N2" s="60" t="s">
+      <c r="K2" s="61"/>
+      <c r="L2" s="61"/>
+      <c r="N2" s="61" t="s">
         <v>132</v>
       </c>
-      <c r="O2" s="60"/>
-      <c r="P2" s="60"/>
-      <c r="R2" s="60" t="s">
+      <c r="O2" s="61"/>
+      <c r="P2" s="61"/>
+      <c r="R2" s="61" t="s">
         <v>133</v>
       </c>
-      <c r="S2" s="60"/>
-      <c r="T2" s="60"/>
-      <c r="V2" s="60" t="s">
+      <c r="S2" s="61"/>
+      <c r="T2" s="61"/>
+      <c r="V2" s="61" t="s">
         <v>134</v>
       </c>
-      <c r="W2" s="60"/>
-      <c r="X2" s="60"/>
+      <c r="W2" s="61"/>
+      <c r="X2" s="61"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -12440,34 +13676,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="62" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="61"/>
-      <c r="E2" s="57" t="s">
+      <c r="C2" s="62"/>
+      <c r="E2" s="58" t="s">
         <v>215</v>
       </c>
-      <c r="F2" s="57"/>
-      <c r="H2" s="57" t="s">
+      <c r="F2" s="58"/>
+      <c r="H2" s="58" t="s">
         <v>217</v>
       </c>
-      <c r="I2" s="57"/>
-      <c r="K2" s="57" t="s">
+      <c r="I2" s="58"/>
+      <c r="K2" s="58" t="s">
         <v>218</v>
       </c>
-      <c r="L2" s="57"/>
-      <c r="N2" s="57" t="s">
+      <c r="L2" s="58"/>
+      <c r="N2" s="58" t="s">
         <v>219</v>
       </c>
-      <c r="O2" s="57"/>
-      <c r="Q2" s="57" t="s">
+      <c r="O2" s="58"/>
+      <c r="Q2" s="58" t="s">
         <v>220</v>
       </c>
-      <c r="R2" s="57"/>
+      <c r="R2" s="58"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
       <c r="E3" s="32" t="s">
         <v>213</v>
       </c>
@@ -12856,34 +14092,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="63" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="E2" s="58" t="s">
+      <c r="C2" s="63"/>
+      <c r="E2" s="59" t="s">
         <v>221</v>
       </c>
-      <c r="F2" s="58"/>
-      <c r="H2" s="58" t="s">
+      <c r="F2" s="59"/>
+      <c r="H2" s="59" t="s">
         <v>222</v>
       </c>
-      <c r="I2" s="58"/>
-      <c r="K2" s="58" t="s">
+      <c r="I2" s="59"/>
+      <c r="K2" s="59" t="s">
         <v>223</v>
       </c>
-      <c r="L2" s="58"/>
-      <c r="N2" s="58" t="s">
+      <c r="L2" s="59"/>
+      <c r="N2" s="59" t="s">
         <v>224</v>
       </c>
-      <c r="O2" s="58"/>
-      <c r="Q2" s="58" t="s">
+      <c r="O2" s="59"/>
+      <c r="Q2" s="59" t="s">
         <v>225</v>
       </c>
-      <c r="R2" s="58"/>
+      <c r="R2" s="59"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
       <c r="E3" s="34" t="s">
         <v>213</v>
       </c>
@@ -13256,6 +14492,939 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B20D353C-FC33-C347-9989-88B2E3FC7B94}">
+  <dimension ref="B2:J100"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="3.5" customWidth="1"/>
+    <col min="2" max="7" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="7.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B2" s="50" t="s">
+        <v>255</v>
+      </c>
+      <c r="C2" s="50" t="s">
+        <v>250</v>
+      </c>
+      <c r="D2" s="50" t="s">
+        <v>251</v>
+      </c>
+      <c r="E2" s="50" t="s">
+        <v>252</v>
+      </c>
+      <c r="F2" s="50" t="s">
+        <v>253</v>
+      </c>
+      <c r="G2" s="50" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="I3" s="14" t="s">
+        <v>257</v>
+      </c>
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="I5" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="I7" s="14" t="s">
+        <v>258</v>
+      </c>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="I8" s="14" t="s">
+        <v>259</v>
+      </c>
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="J10" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="J11" s="4"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="J12" s="4"/>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="J13" s="4"/>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="J14" s="4"/>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="J15" s="4"/>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="J16" s="4"/>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="J17" s="4"/>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="J18" s="4"/>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="J19" s="4"/>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="J20" s="4"/>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="J21" s="4"/>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="J22" s="4"/>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="J23" s="4"/>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="J24" s="4"/>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="J25" s="4"/>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="J26" s="4"/>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="J27" s="4"/>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="J28" s="4"/>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="J29" s="4"/>
+    </row>
+    <row r="30" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="J30" s="4"/>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="J31" s="4"/>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="J32" s="4"/>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="J33" s="4"/>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="J34" s="4"/>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="J35" s="4"/>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="J36" s="4"/>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="J37" s="4"/>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="J38" s="4"/>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="J39" s="4"/>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="J40" s="4"/>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="J41" s="4"/>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="J42" s="4"/>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="J43" s="4"/>
+    </row>
+    <row r="44" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="J44" s="4"/>
+    </row>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="J45" s="4"/>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="J46" s="4"/>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="J47" s="4"/>
+    </row>
+    <row r="48" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="J48" s="4"/>
+    </row>
+    <row r="49" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="J49" s="4"/>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="J50" s="4"/>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="J51" s="4"/>
+    </row>
+    <row r="52" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="J52" s="4"/>
+    </row>
+    <row r="53" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="J53" s="4"/>
+    </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B54" s="3"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="J54" s="4"/>
+    </row>
+    <row r="55" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="J55" s="4"/>
+    </row>
+    <row r="56" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B56" s="3"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="J56" s="4"/>
+    </row>
+    <row r="57" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="J57" s="4"/>
+    </row>
+    <row r="58" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B58" s="3"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="J58" s="4"/>
+    </row>
+    <row r="59" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B59" s="3"/>
+      <c r="C59" s="3"/>
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="J59" s="4"/>
+    </row>
+    <row r="60" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B60" s="3"/>
+      <c r="C60" s="3"/>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="J60" s="4"/>
+    </row>
+    <row r="61" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B61" s="3"/>
+      <c r="C61" s="3"/>
+      <c r="D61" s="3"/>
+      <c r="E61" s="3"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="J61" s="4"/>
+    </row>
+    <row r="62" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B62" s="3"/>
+      <c r="C62" s="3"/>
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="J62" s="4"/>
+    </row>
+    <row r="63" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B63" s="3"/>
+      <c r="C63" s="3"/>
+      <c r="D63" s="3"/>
+      <c r="E63" s="3"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+      <c r="J63" s="4"/>
+    </row>
+    <row r="64" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B64" s="3"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
+      <c r="J64" s="4"/>
+    </row>
+    <row r="65" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B65" s="3"/>
+      <c r="C65" s="3"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="3"/>
+      <c r="G65" s="3"/>
+      <c r="J65" s="4"/>
+    </row>
+    <row r="66" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B66" s="3"/>
+      <c r="C66" s="3"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
+      <c r="J66" s="4"/>
+    </row>
+    <row r="67" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B67" s="3"/>
+      <c r="C67" s="3"/>
+      <c r="D67" s="3"/>
+      <c r="E67" s="3"/>
+      <c r="F67" s="3"/>
+      <c r="G67" s="3"/>
+      <c r="J67" s="4"/>
+    </row>
+    <row r="68" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B68" s="3"/>
+      <c r="C68" s="3"/>
+      <c r="D68" s="3"/>
+      <c r="E68" s="3"/>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+      <c r="J68" s="4"/>
+    </row>
+    <row r="69" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B69" s="3"/>
+      <c r="C69" s="3"/>
+      <c r="D69" s="3"/>
+      <c r="E69" s="3"/>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+      <c r="J69" s="4"/>
+    </row>
+    <row r="70" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B70" s="3"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3"/>
+      <c r="E70" s="3"/>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
+      <c r="J70" s="4"/>
+    </row>
+    <row r="71" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B71" s="3"/>
+      <c r="C71" s="3"/>
+      <c r="D71" s="3"/>
+      <c r="E71" s="3"/>
+      <c r="F71" s="3"/>
+      <c r="G71" s="3"/>
+      <c r="J71" s="4"/>
+    </row>
+    <row r="72" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B72" s="3"/>
+      <c r="C72" s="3"/>
+      <c r="D72" s="3"/>
+      <c r="E72" s="3"/>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
+      <c r="J72" s="4"/>
+    </row>
+    <row r="73" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B73" s="3"/>
+      <c r="C73" s="3"/>
+      <c r="D73" s="3"/>
+      <c r="E73" s="3"/>
+      <c r="F73" s="3"/>
+      <c r="G73" s="3"/>
+      <c r="J73" s="4"/>
+    </row>
+    <row r="74" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B74" s="3"/>
+      <c r="C74" s="3"/>
+      <c r="D74" s="3"/>
+      <c r="E74" s="3"/>
+      <c r="F74" s="3"/>
+      <c r="G74" s="3"/>
+      <c r="J74" s="4"/>
+    </row>
+    <row r="75" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B75" s="3"/>
+      <c r="C75" s="3"/>
+      <c r="D75" s="3"/>
+      <c r="E75" s="3"/>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3"/>
+      <c r="J75" s="4"/>
+    </row>
+    <row r="76" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B76" s="3"/>
+      <c r="C76" s="3"/>
+      <c r="D76" s="3"/>
+      <c r="E76" s="3"/>
+      <c r="F76" s="3"/>
+      <c r="G76" s="3"/>
+      <c r="J76" s="4"/>
+    </row>
+    <row r="77" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B77" s="3"/>
+      <c r="C77" s="3"/>
+      <c r="D77" s="3"/>
+      <c r="E77" s="3"/>
+      <c r="F77" s="3"/>
+      <c r="G77" s="3"/>
+      <c r="J77" s="4"/>
+    </row>
+    <row r="78" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B78" s="3"/>
+      <c r="C78" s="3"/>
+      <c r="D78" s="3"/>
+      <c r="E78" s="3"/>
+      <c r="F78" s="3"/>
+      <c r="G78" s="3"/>
+      <c r="J78" s="4"/>
+    </row>
+    <row r="79" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B79" s="3"/>
+      <c r="C79" s="3"/>
+      <c r="D79" s="3"/>
+      <c r="E79" s="3"/>
+      <c r="F79" s="3"/>
+      <c r="G79" s="3"/>
+      <c r="J79" s="4"/>
+    </row>
+    <row r="80" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B80" s="3"/>
+      <c r="C80" s="3"/>
+      <c r="D80" s="3"/>
+      <c r="E80" s="3"/>
+      <c r="F80" s="3"/>
+      <c r="G80" s="3"/>
+      <c r="J80" s="4"/>
+    </row>
+    <row r="81" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B81" s="3"/>
+      <c r="C81" s="3"/>
+      <c r="D81" s="3"/>
+      <c r="E81" s="3"/>
+      <c r="F81" s="3"/>
+      <c r="G81" s="3"/>
+      <c r="J81" s="4"/>
+    </row>
+    <row r="82" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B82" s="3"/>
+      <c r="C82" s="3"/>
+      <c r="D82" s="3"/>
+      <c r="E82" s="3"/>
+      <c r="F82" s="3"/>
+      <c r="G82" s="3"/>
+      <c r="J82" s="4"/>
+    </row>
+    <row r="83" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B83" s="3"/>
+      <c r="C83" s="3"/>
+      <c r="D83" s="3"/>
+      <c r="E83" s="3"/>
+      <c r="F83" s="3"/>
+      <c r="G83" s="3"/>
+      <c r="J83" s="4"/>
+    </row>
+    <row r="84" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B84" s="3"/>
+      <c r="C84" s="3"/>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
+      <c r="F84" s="3"/>
+      <c r="G84" s="3"/>
+      <c r="J84" s="4"/>
+    </row>
+    <row r="85" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B85" s="3"/>
+      <c r="C85" s="3"/>
+      <c r="D85" s="3"/>
+      <c r="E85" s="3"/>
+      <c r="F85" s="3"/>
+      <c r="G85" s="3"/>
+      <c r="J85" s="4"/>
+    </row>
+    <row r="86" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B86" s="3"/>
+      <c r="C86" s="3"/>
+      <c r="D86" s="3"/>
+      <c r="E86" s="3"/>
+      <c r="F86" s="3"/>
+      <c r="G86" s="3"/>
+      <c r="J86" s="4"/>
+    </row>
+    <row r="87" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B87" s="3"/>
+      <c r="C87" s="3"/>
+      <c r="D87" s="3"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+      <c r="G87" s="3"/>
+      <c r="J87" s="4"/>
+    </row>
+    <row r="88" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B88" s="3"/>
+      <c r="C88" s="3"/>
+      <c r="D88" s="3"/>
+      <c r="E88" s="3"/>
+      <c r="F88" s="3"/>
+      <c r="G88" s="3"/>
+      <c r="J88" s="4"/>
+    </row>
+    <row r="89" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B89" s="3"/>
+      <c r="C89" s="3"/>
+      <c r="D89" s="3"/>
+      <c r="E89" s="3"/>
+      <c r="F89" s="3"/>
+      <c r="G89" s="3"/>
+      <c r="J89" s="4"/>
+    </row>
+    <row r="90" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B90" s="3"/>
+      <c r="C90" s="3"/>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3"/>
+      <c r="G90" s="3"/>
+      <c r="J90" s="4"/>
+    </row>
+    <row r="91" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B91" s="3"/>
+      <c r="C91" s="3"/>
+      <c r="D91" s="3"/>
+      <c r="E91" s="3"/>
+      <c r="F91" s="3"/>
+      <c r="G91" s="3"/>
+      <c r="J91" s="4"/>
+    </row>
+    <row r="92" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B92" s="3"/>
+      <c r="C92" s="3"/>
+      <c r="D92" s="3"/>
+      <c r="E92" s="3"/>
+      <c r="F92" s="3"/>
+      <c r="G92" s="3"/>
+      <c r="J92" s="4"/>
+    </row>
+    <row r="93" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B93" s="3"/>
+      <c r="C93" s="3"/>
+      <c r="D93" s="3"/>
+      <c r="E93" s="3"/>
+      <c r="F93" s="3"/>
+      <c r="G93" s="3"/>
+      <c r="J93" s="4"/>
+    </row>
+    <row r="94" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B94" s="3"/>
+      <c r="C94" s="3"/>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3"/>
+      <c r="G94" s="3"/>
+      <c r="J94" s="4"/>
+    </row>
+    <row r="95" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B95" s="3"/>
+      <c r="C95" s="3"/>
+      <c r="D95" s="3"/>
+      <c r="E95" s="3"/>
+      <c r="F95" s="3"/>
+      <c r="G95" s="3"/>
+      <c r="J95" s="4"/>
+    </row>
+    <row r="96" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B96" s="3"/>
+      <c r="C96" s="3"/>
+      <c r="D96" s="3"/>
+      <c r="E96" s="3"/>
+      <c r="F96" s="3"/>
+      <c r="G96" s="3"/>
+      <c r="J96" s="4"/>
+    </row>
+    <row r="97" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B97" s="3"/>
+      <c r="C97" s="3"/>
+      <c r="D97" s="3"/>
+      <c r="E97" s="3"/>
+      <c r="F97" s="3"/>
+      <c r="G97" s="3"/>
+      <c r="J97" s="4"/>
+    </row>
+    <row r="98" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B98" s="3"/>
+      <c r="C98" s="3"/>
+      <c r="D98" s="3"/>
+      <c r="E98" s="3"/>
+      <c r="F98" s="3"/>
+      <c r="G98" s="3"/>
+      <c r="J98" s="4"/>
+    </row>
+    <row r="99" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B99" s="3"/>
+      <c r="C99" s="3"/>
+      <c r="D99" s="3"/>
+      <c r="E99" s="3"/>
+      <c r="F99" s="3"/>
+      <c r="G99" s="3"/>
+      <c r="J99" s="4"/>
+    </row>
+    <row r="100" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B100" s="3"/>
+      <c r="C100" s="3"/>
+      <c r="D100" s="3"/>
+      <c r="E100" s="3"/>
+      <c r="F100" s="3"/>
+      <c r="G100" s="3"/>
+      <c r="J100" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDB4949D-EAAF-AE4C-9BAF-D5BF753E34CD}">
   <dimension ref="A1"/>
@@ -13268,16 +15437,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A900FC-A692-B445-95C9-59E70352B291}">
-  <dimension ref="A2:AN52"/>
+  <dimension ref="A2:AP52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
     <col min="3" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="40" width="8.5" customWidth="1"/>
+    <col min="11" max="42" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
         <v>67</v>
       </c>
@@ -13295,7 +15464,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
         <v>66</v>
       </c>
@@ -13318,7 +15487,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="4" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
         <v>69</v>
       </c>
@@ -13345,7 +15514,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="5" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C5" s="1" t="s">
         <v>171</v>
       </c>
@@ -13370,7 +15539,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="6" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C6" s="1" t="s">
         <v>201</v>
       </c>
@@ -13390,7 +15559,7 @@
       <c r="AE6" s="1"/>
       <c r="AF6" s="1"/>
     </row>
-    <row r="7" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C7" s="1" t="s">
         <v>233</v>
       </c>
@@ -13400,53 +15569,55 @@
       <c r="AE7" s="1"/>
       <c r="AF7" s="1"/>
     </row>
-    <row r="9" spans="1:40" x14ac:dyDescent="0.2">
-      <c r="C9" s="51" t="s">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="C9" s="52" t="s">
         <v>236</v>
       </c>
-      <c r="D9" s="51"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="51"/>
-      <c r="G9" s="51"/>
-      <c r="H9" s="51"/>
-      <c r="I9" s="51"/>
-      <c r="J9" s="51"/>
-      <c r="K9" s="51"/>
-      <c r="L9" s="51"/>
-      <c r="M9" s="51"/>
-      <c r="N9" s="51"/>
-      <c r="O9" s="51"/>
-      <c r="P9" s="51"/>
-      <c r="Q9" s="51"/>
-      <c r="R9" s="51"/>
-      <c r="S9" s="51"/>
-      <c r="T9" s="51"/>
-      <c r="U9" s="51"/>
-      <c r="V9" s="51"/>
-      <c r="W9" s="51"/>
-      <c r="X9" s="51"/>
-      <c r="Y9" s="51"/>
-      <c r="Z9" s="51"/>
-      <c r="AA9" s="51" t="s">
+      <c r="D9" s="52"/>
+      <c r="E9" s="52"/>
+      <c r="F9" s="52"/>
+      <c r="G9" s="52"/>
+      <c r="H9" s="52"/>
+      <c r="I9" s="52"/>
+      <c r="J9" s="52"/>
+      <c r="K9" s="52"/>
+      <c r="L9" s="52"/>
+      <c r="M9" s="52"/>
+      <c r="N9" s="52"/>
+      <c r="O9" s="52"/>
+      <c r="P9" s="52"/>
+      <c r="Q9" s="52"/>
+      <c r="R9" s="52"/>
+      <c r="S9" s="52"/>
+      <c r="T9" s="52"/>
+      <c r="U9" s="52"/>
+      <c r="V9" s="52"/>
+      <c r="W9" s="52"/>
+      <c r="X9" s="52"/>
+      <c r="Y9" s="52"/>
+      <c r="Z9" s="52"/>
+      <c r="AA9" s="52" t="s">
         <v>57</v>
       </c>
-      <c r="AB9" s="51"/>
-      <c r="AC9" s="51"/>
-      <c r="AD9" s="51"/>
-      <c r="AE9" s="51"/>
-      <c r="AF9" s="51"/>
-      <c r="AG9" s="51" t="s">
+      <c r="AB9" s="52"/>
+      <c r="AC9" s="52"/>
+      <c r="AD9" s="52"/>
+      <c r="AE9" s="52"/>
+      <c r="AF9" s="52"/>
+      <c r="AG9" s="52" t="s">
         <v>91</v>
       </c>
-      <c r="AH9" s="51"/>
-      <c r="AI9" s="51"/>
-      <c r="AJ9" s="51"/>
-      <c r="AK9" s="51"/>
-      <c r="AL9" s="51"/>
-      <c r="AM9" s="51"/>
-      <c r="AN9" s="51"/>
-    </row>
-    <row r="10" spans="1:40" ht="18" x14ac:dyDescent="0.25">
+      <c r="AH9" s="52"/>
+      <c r="AI9" s="52"/>
+      <c r="AJ9" s="52"/>
+      <c r="AK9" s="52"/>
+      <c r="AL9" s="52"/>
+      <c r="AM9" s="52"/>
+      <c r="AN9" s="52"/>
+      <c r="AO9" s="52"/>
+      <c r="AP9" s="52"/>
+    </row>
+    <row r="10" spans="1:42" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
         <v>19</v>
       </c>
@@ -13567,8 +15738,14 @@
       <c r="AN10" s="23" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="11" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO10" s="23" t="s">
+        <v>262</v>
+      </c>
+      <c r="AP10" s="23" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="11" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>1</v>
       </c>
@@ -13611,8 +15788,10 @@
       <c r="AL11" s="3"/>
       <c r="AM11" s="3"/>
       <c r="AN11" s="3"/>
-    </row>
-    <row r="12" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO11" s="3"/>
+      <c r="AP11" s="3"/>
+    </row>
+    <row r="12" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -13655,8 +15834,10 @@
       <c r="AL12" s="3"/>
       <c r="AM12" s="18"/>
       <c r="AN12" s="19"/>
-    </row>
-    <row r="13" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO12" s="19"/>
+      <c r="AP12" s="19"/>
+    </row>
+    <row r="13" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>3</v>
       </c>
@@ -13699,8 +15880,10 @@
       <c r="AL13" s="3"/>
       <c r="AM13" s="18"/>
       <c r="AN13" s="19"/>
-    </row>
-    <row r="14" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO13" s="19"/>
+      <c r="AP13" s="19"/>
+    </row>
+    <row r="14" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>4</v>
       </c>
@@ -13743,8 +15926,10 @@
       <c r="AL14" s="3"/>
       <c r="AM14" s="3"/>
       <c r="AN14" s="3"/>
-    </row>
-    <row r="15" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO14" s="3"/>
+      <c r="AP14" s="3"/>
+    </row>
+    <row r="15" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>5</v>
       </c>
@@ -13787,8 +15972,10 @@
       <c r="AL15" s="3"/>
       <c r="AM15" s="3"/>
       <c r="AN15" s="3"/>
-    </row>
-    <row r="16" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO15" s="3"/>
+      <c r="AP15" s="3"/>
+    </row>
+    <row r="16" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>6</v>
       </c>
@@ -13831,8 +16018,10 @@
       <c r="AL16" s="3"/>
       <c r="AM16" s="3"/>
       <c r="AN16" s="3"/>
-    </row>
-    <row r="17" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO16" s="3"/>
+      <c r="AP16" s="3"/>
+    </row>
+    <row r="17" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>7</v>
       </c>
@@ -13875,8 +16064,10 @@
       <c r="AL17" s="3"/>
       <c r="AM17" s="3"/>
       <c r="AN17" s="3"/>
-    </row>
-    <row r="18" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO17" s="3"/>
+      <c r="AP17" s="3"/>
+    </row>
+    <row r="18" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>8</v>
       </c>
@@ -13919,8 +16110,10 @@
       <c r="AL18" s="3"/>
       <c r="AM18" s="3"/>
       <c r="AN18" s="3"/>
-    </row>
-    <row r="19" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO18" s="3"/>
+      <c r="AP18" s="3"/>
+    </row>
+    <row r="19" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>9</v>
       </c>
@@ -13963,8 +16156,10 @@
       <c r="AL19" s="3"/>
       <c r="AM19" s="3"/>
       <c r="AN19" s="3"/>
-    </row>
-    <row r="20" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO19" s="3"/>
+      <c r="AP19" s="3"/>
+    </row>
+    <row r="20" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>10</v>
       </c>
@@ -14007,8 +16202,10 @@
       <c r="AL20" s="3"/>
       <c r="AM20" s="3"/>
       <c r="AN20" s="3"/>
-    </row>
-    <row r="21" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO20" s="3"/>
+      <c r="AP20" s="3"/>
+    </row>
+    <row r="21" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>11</v>
       </c>
@@ -14051,8 +16248,10 @@
       <c r="AL21" s="3"/>
       <c r="AM21" s="3"/>
       <c r="AN21" s="3"/>
-    </row>
-    <row r="22" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO21" s="3"/>
+      <c r="AP21" s="3"/>
+    </row>
+    <row r="22" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>12</v>
       </c>
@@ -14095,8 +16294,10 @@
       <c r="AL22" s="3"/>
       <c r="AM22" s="3"/>
       <c r="AN22" s="3"/>
-    </row>
-    <row r="23" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO22" s="3"/>
+      <c r="AP22" s="3"/>
+    </row>
+    <row r="23" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>13</v>
       </c>
@@ -14139,8 +16340,10 @@
       <c r="AL23" s="3"/>
       <c r="AM23" s="3"/>
       <c r="AN23" s="3"/>
-    </row>
-    <row r="24" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO23" s="3"/>
+      <c r="AP23" s="3"/>
+    </row>
+    <row r="24" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>14</v>
       </c>
@@ -14183,8 +16386,10 @@
       <c r="AL24" s="3"/>
       <c r="AM24" s="3"/>
       <c r="AN24" s="3"/>
-    </row>
-    <row r="25" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO24" s="3"/>
+      <c r="AP24" s="3"/>
+    </row>
+    <row r="25" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>15</v>
       </c>
@@ -14227,8 +16432,10 @@
       <c r="AL25" s="3"/>
       <c r="AM25" s="3"/>
       <c r="AN25" s="3"/>
-    </row>
-    <row r="26" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO25" s="3"/>
+      <c r="AP25" s="3"/>
+    </row>
+    <row r="26" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -14259,8 +16466,10 @@
       <c r="AL26" s="1"/>
       <c r="AM26" s="1"/>
       <c r="AN26" s="1"/>
-    </row>
-    <row r="27" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO26" s="1"/>
+      <c r="AP26" s="1"/>
+    </row>
+    <row r="27" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -14284,7 +16493,7 @@
       <c r="AE27" s="1"/>
       <c r="AF27" s="1"/>
     </row>
-    <row r="28" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -14308,7 +16517,7 @@
       <c r="AE28" s="1"/>
       <c r="AF28" s="1"/>
     </row>
-    <row r="29" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -14332,7 +16541,7 @@
       <c r="AE29" s="1"/>
       <c r="AF29" s="1"/>
     </row>
-    <row r="30" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -14356,7 +16565,7 @@
       <c r="AE30" s="1"/>
       <c r="AF30" s="1"/>
     </row>
-    <row r="31" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -14380,7 +16589,7 @@
       <c r="AE31" s="1"/>
       <c r="AF31" s="1"/>
     </row>
-    <row r="32" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -14887,100 +17096,93 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="AA9:AF9"/>
-    <mergeCell ref="AG9:AN9"/>
     <mergeCell ref="C9:Z9"/>
+    <mergeCell ref="AG9:AP9"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:K52 AB11:AF52">
-    <cfRule type="expression" dxfId="21" priority="4">
+    <cfRule type="expression" dxfId="20" priority="6">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="5">
+    <cfRule type="expression" dxfId="19" priority="7">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11:L52">
-    <cfRule type="expression" dxfId="19" priority="17">
+    <cfRule type="expression" dxfId="18" priority="19">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="18" priority="6">
+    <cfRule type="expression" dxfId="17" priority="8">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="17" priority="7">
+    <cfRule type="expression" dxfId="16" priority="9">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="16" priority="8">
+    <cfRule type="expression" dxfId="15" priority="10">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O11:P52">
-    <cfRule type="expression" dxfId="15" priority="18">
+  <conditionalFormatting sqref="O11:R52">
+    <cfRule type="expression" dxfId="14" priority="4">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P11:P52">
-    <cfRule type="expression" dxfId="14" priority="11">
+    <cfRule type="expression" dxfId="13" priority="13">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="12" priority="3">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="11" priority="5">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="S11:V52">
-    <cfRule type="expression" dxfId="13" priority="9">
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W11:Z52">
-    <cfRule type="expression" dxfId="12" priority="10">
+    <cfRule type="expression" dxfId="9" priority="12">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB11:AF52">
-    <cfRule type="expression" dxfId="11" priority="19">
+    <cfRule type="expression" dxfId="8" priority="21">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC11:AC52">
-    <cfRule type="expression" dxfId="10" priority="12">
+    <cfRule type="expression" dxfId="7" priority="14">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="9" priority="13">
+    <cfRule type="expression" dxfId="6" priority="15">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE11:AF52">
-    <cfRule type="expression" dxfId="8" priority="14">
+    <cfRule type="expression" dxfId="5" priority="16">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="7" priority="15">
+    <cfRule type="expression" dxfId="4" priority="17">
       <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM11:AN52">
-    <cfRule type="expression" dxfId="6" priority="16">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$AJ11="lf"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="5" priority="2">
-      <formula>$E11="elastic"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="4" priority="1">
-      <formula>$E11="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="3" priority="3">
-      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -15036,74 +17238,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="55"/>
+      <c r="D4" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="54"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="55"/>
+      <c r="G4" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="54"/>
-      <c r="J4" s="54" t="s">
+      <c r="H4" s="55"/>
+      <c r="J4" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="54"/>
-      <c r="M4" s="54" t="s">
+      <c r="K4" s="55"/>
+      <c r="M4" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="54"/>
-      <c r="P4" s="54" t="s">
+      <c r="N4" s="55"/>
+      <c r="P4" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="54"/>
+      <c r="Q4" s="55"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="54" t="s">
+      <c r="S4" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="54"/>
+      <c r="T4" s="55"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="54" t="s">
+      <c r="V4" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="54"/>
+      <c r="W4" s="55"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="54" t="s">
+      <c r="Y4" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="54"/>
+      <c r="Z4" s="55"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="54" t="s">
+      <c r="AB4" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="54"/>
-      <c r="AE4" s="54" t="s">
+      <c r="AC4" s="55"/>
+      <c r="AE4" s="55" t="s">
         <v>108</v>
       </c>
-      <c r="AF4" s="54"/>
+      <c r="AF4" s="55"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="54" t="s">
+      <c r="AH4" s="55" t="s">
         <v>109</v>
       </c>
-      <c r="AI4" s="54"/>
+      <c r="AI4" s="55"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="54" t="s">
+      <c r="AK4" s="55" t="s">
         <v>110</v>
       </c>
-      <c r="AL4" s="54"/>
+      <c r="AL4" s="55"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="54" t="s">
+      <c r="AN4" s="55" t="s">
         <v>111</v>
       </c>
-      <c r="AO4" s="54"/>
+      <c r="AO4" s="55"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="54" t="s">
+      <c r="AQ4" s="55" t="s">
         <v>112</v>
       </c>
-      <c r="AR4" s="54"/>
+      <c r="AR4" s="55"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
@@ -15206,89 +17408,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="52" t="str">
+      <c r="A6" s="53" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="53"/>
-      <c r="D6" s="52" t="str">
+      <c r="B6" s="54"/>
+      <c r="D6" s="53" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="53"/>
-      <c r="G6" s="52" t="str">
+      <c r="E6" s="54"/>
+      <c r="G6" s="53" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="53"/>
-      <c r="J6" s="52" t="str">
+      <c r="H6" s="54"/>
+      <c r="J6" s="53" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="53"/>
-      <c r="M6" s="52" t="str">
+      <c r="K6" s="54"/>
+      <c r="M6" s="53" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="53"/>
-      <c r="P6" s="52" t="str">
+      <c r="N6" s="54"/>
+      <c r="P6" s="53" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="53"/>
+      <c r="Q6" s="54"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="52" t="str">
+      <c r="S6" s="53" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="53"/>
+      <c r="T6" s="54"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="52" t="str">
+      <c r="V6" s="53" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="53"/>
+      <c r="W6" s="54"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="52" t="str">
+      <c r="Y6" s="53" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="53"/>
+      <c r="Z6" s="54"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="52" t="str">
+      <c r="AB6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="53"/>
-      <c r="AE6" s="52" t="str">
+      <c r="AC6" s="54"/>
+      <c r="AE6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="53"/>
+      <c r="AF6" s="54"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="52" t="str">
+      <c r="AH6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="53"/>
+      <c r="AI6" s="54"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="52" t="str">
+      <c r="AK6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="53"/>
+      <c r="AL6" s="54"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="52" t="str">
+      <c r="AN6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="53"/>
+      <c r="AO6" s="54"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="52" t="str">
+      <c r="AQ6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="53"/>
+      <c r="AR6" s="54"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -16259,74 +18461,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="55" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="55"/>
+      <c r="D4" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="E4" s="54"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="55"/>
+      <c r="G4" s="55" t="s">
         <v>139</v>
       </c>
-      <c r="H4" s="54"/>
-      <c r="J4" s="54" t="s">
+      <c r="H4" s="55"/>
+      <c r="J4" s="55" t="s">
         <v>140</v>
       </c>
-      <c r="K4" s="54"/>
-      <c r="M4" s="54" t="s">
+      <c r="K4" s="55"/>
+      <c r="M4" s="55" t="s">
         <v>141</v>
       </c>
-      <c r="N4" s="54"/>
-      <c r="P4" s="54" t="s">
+      <c r="N4" s="55"/>
+      <c r="P4" s="55" t="s">
         <v>142</v>
       </c>
-      <c r="Q4" s="54"/>
+      <c r="Q4" s="55"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="54" t="s">
+      <c r="S4" s="55" t="s">
         <v>143</v>
       </c>
-      <c r="T4" s="54"/>
+      <c r="T4" s="55"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="54" t="s">
+      <c r="V4" s="55" t="s">
         <v>144</v>
       </c>
-      <c r="W4" s="54"/>
+      <c r="W4" s="55"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="54" t="s">
+      <c r="Y4" s="55" t="s">
         <v>145</v>
       </c>
-      <c r="Z4" s="54"/>
+      <c r="Z4" s="55"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="54" t="s">
+      <c r="AB4" s="55" t="s">
         <v>146</v>
       </c>
-      <c r="AC4" s="54"/>
-      <c r="AE4" s="54" t="s">
+      <c r="AC4" s="55"/>
+      <c r="AE4" s="55" t="s">
         <v>147</v>
       </c>
-      <c r="AF4" s="54"/>
+      <c r="AF4" s="55"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="54" t="s">
+      <c r="AH4" s="55" t="s">
         <v>148</v>
       </c>
-      <c r="AI4" s="54"/>
+      <c r="AI4" s="55"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="54" t="s">
+      <c r="AK4" s="55" t="s">
         <v>149</v>
       </c>
-      <c r="AL4" s="54"/>
+      <c r="AL4" s="55"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="54" t="s">
+      <c r="AN4" s="55" t="s">
         <v>150</v>
       </c>
-      <c r="AO4" s="54"/>
+      <c r="AO4" s="55"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="54" t="s">
+      <c r="AQ4" s="55" t="s">
         <v>151</v>
       </c>
-      <c r="AR4" s="54"/>
+      <c r="AR4" s="55"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
@@ -16429,89 +18631,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="55" t="str">
+      <c r="A6" s="56" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="56"/>
-      <c r="D6" s="55" t="str">
+      <c r="B6" s="57"/>
+      <c r="D6" s="56" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="56"/>
-      <c r="G6" s="55" t="str">
+      <c r="E6" s="57"/>
+      <c r="G6" s="56" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="56"/>
-      <c r="J6" s="55" t="str">
+      <c r="H6" s="57"/>
+      <c r="J6" s="56" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="56"/>
-      <c r="M6" s="55" t="str">
+      <c r="K6" s="57"/>
+      <c r="M6" s="56" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="56"/>
-      <c r="P6" s="55" t="str">
+      <c r="N6" s="57"/>
+      <c r="P6" s="56" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="56"/>
+      <c r="Q6" s="57"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="55" t="str">
+      <c r="S6" s="56" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="56"/>
+      <c r="T6" s="57"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="55" t="str">
+      <c r="V6" s="56" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="56"/>
+      <c r="W6" s="57"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="55" t="str">
+      <c r="Y6" s="56" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="56"/>
+      <c r="Z6" s="57"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="55" t="str">
+      <c r="AB6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="56"/>
-      <c r="AE6" s="55" t="str">
+      <c r="AC6" s="57"/>
+      <c r="AE6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="56"/>
+      <c r="AF6" s="57"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="55" t="str">
+      <c r="AH6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="56"/>
+      <c r="AI6" s="57"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="55" t="str">
+      <c r="AK6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="56"/>
+      <c r="AL6" s="57"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="55" t="str">
+      <c r="AN6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="56"/>
+      <c r="AO6" s="57"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="55" t="str">
+      <c r="AQ6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="56"/>
+      <c r="AR6" s="57"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -17460,14 +19662,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="58" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="57"/>
-      <c r="D2" s="58" t="s">
+      <c r="B2" s="58"/>
+      <c r="D2" s="59" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="58"/>
+      <c r="E2" s="59"/>
       <c r="G2" s="22" t="s">
         <v>82</v>
       </c>
@@ -18038,36 +20240,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="60" t="s">
         <v>121</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="F2" s="59" t="s">
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="F2" s="60" t="s">
         <v>122</v>
       </c>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="J2" s="59" t="s">
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="J2" s="60" t="s">
         <v>123</v>
       </c>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="N2" s="59" t="s">
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="N2" s="60" t="s">
         <v>124</v>
       </c>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="R2" s="59" t="s">
+      <c r="O2" s="60"/>
+      <c r="P2" s="60"/>
+      <c r="R2" s="60" t="s">
         <v>125</v>
       </c>
-      <c r="S2" s="59"/>
-      <c r="T2" s="59"/>
-      <c r="V2" s="59" t="s">
+      <c r="S2" s="60"/>
+      <c r="T2" s="60"/>
+      <c r="V2" s="60" t="s">
         <v>126</v>
       </c>
-      <c r="W2" s="59"/>
-      <c r="X2" s="59"/>
+      <c r="W2" s="60"/>
+      <c r="X2" s="60"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">

</xml_diff>